<commit_message>
Slideshow back up and running.
</commit_message>
<xml_diff>
--- a/pm2022/pm2022.xlsx
+++ b/pm2022/pm2022.xlsx
@@ -49,7 +49,7 @@
     <t xml:space="preserve">Detector Systems and Future accelerators</t>
   </si>
   <si>
-    <t xml:space="preserve">23/05/2022 10:20</t>
+    <t xml:space="preserve">23/05/2021 10:20</t>
   </si>
   <si>
     <t xml:space="preserve">23/05/2022 12:40</t>
@@ -61,7 +61,7 @@
     <t xml:space="preserve">Photo Detectors and PID</t>
   </si>
   <si>
-    <t xml:space="preserve">23/05/2022 15:30</t>
+    <t xml:space="preserve">23/05/2021 15:30</t>
   </si>
   <si>
     <t xml:space="preserve">23/05/2022 18:50</t>
@@ -73,7 +73,7 @@
     <t xml:space="preserve">Solid State Detectors</t>
   </si>
   <si>
-    <t xml:space="preserve">24/05/2021 08:30</t>
+    <t xml:space="preserve">24/05/2022 08:30</t>
   </si>
   <si>
     <t xml:space="preserve">24/05/2022 12:15</t>
@@ -85,7 +85,7 @@
     <t xml:space="preserve">Application to life sciences and other societal challanges</t>
   </si>
   <si>
-    <t xml:space="preserve">24/05/2021 15:30</t>
+    <t xml:space="preserve">24/05/2022 15:30</t>
   </si>
   <si>
     <t xml:space="preserve">24/05/2022 19:10</t>
@@ -3719,7 +3719,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="8.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="100.71"/>
@@ -3868,8 +3868,8 @@
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -3883,7 +3883,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G62"/>
-  <sheetFormatPr defaultColWidth="8.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="12.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="100.71"/>
@@ -5112,8 +5112,8 @@
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -5127,7 +5127,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G22"/>
-  <sheetFormatPr defaultColWidth="8.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="12.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="100.71"/>
@@ -5165,6 +5165,9 @@
       <c r="B2" s="0" t="n">
         <v>166463</v>
       </c>
+      <c r="C2" s="0" t="n">
+        <v>1</v>
+      </c>
       <c r="D2" s="0" t="s">
         <v>48</v>
       </c>
@@ -5182,6 +5185,9 @@
       <c r="B3" s="0" t="n">
         <v>166513</v>
       </c>
+      <c r="C3" s="0" t="n">
+        <v>1</v>
+      </c>
       <c r="D3" s="0" t="s">
         <v>52</v>
       </c>
@@ -5202,6 +5208,9 @@
       <c r="B4" s="0" t="n">
         <v>166553</v>
       </c>
+      <c r="C4" s="0" t="n">
+        <v>1</v>
+      </c>
       <c r="D4" s="0" t="s">
         <v>57</v>
       </c>
@@ -5222,6 +5231,9 @@
       <c r="B5" s="0" t="n">
         <v>166712</v>
       </c>
+      <c r="C5" s="0" t="n">
+        <v>1</v>
+      </c>
       <c r="D5" s="0" t="s">
         <v>62</v>
       </c>
@@ -5565,8 +5577,8 @@
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -5580,7 +5592,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="8.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="12.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="100.71"/>
@@ -5987,8 +5999,8 @@
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -6002,7 +6014,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G55"/>
-  <sheetFormatPr defaultColWidth="8.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="12.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="100.71"/>
@@ -7094,8 +7106,8 @@
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -7109,7 +7121,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G24"/>
-  <sheetFormatPr defaultColWidth="8.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="12.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="100.71"/>
@@ -7599,8 +7611,8 @@
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -7614,7 +7626,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G24"/>
-  <sheetFormatPr defaultColWidth="8.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="12.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="100.71"/>
@@ -8092,8 +8104,8 @@
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -8107,7 +8119,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultColWidth="8.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="12.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="100.71"/>
@@ -8140,8 +8152,8 @@
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -8155,7 +8167,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G46"/>
-  <sheetFormatPr defaultColWidth="8.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="12.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="100.71"/>
@@ -9085,8 +9097,8 @@
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -9100,7 +9112,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G47"/>
-  <sheetFormatPr defaultColWidth="8.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="12.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="100.71"/>
@@ -10041,8 +10053,8 @@
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>

<commit_message>
session with screens and date
</commit_message>
<xml_diff>
--- a/pm2022/pm2022.xlsx
+++ b/pm2022/pm2022.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/galli/Documents/OrgConferenze/21PisaMeeting/pisameet/pm2022/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B718B10-E89A-D645-A20C-3A3398FF4786}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC8F2CDB-704C-354C-9E03-A9EE769BD09B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Program" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1490" uniqueCount="1184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1508" uniqueCount="1194">
   <si>
     <t>Session ID</t>
   </si>
@@ -3581,13 +3581,43 @@
   </si>
   <si>
     <t>Jagiellonian University</t>
+  </si>
+  <si>
+    <t>23/05/22 5:00</t>
+  </si>
+  <si>
+    <t>24/05/22 5:00</t>
+  </si>
+  <si>
+    <t>25/05/22 5:00</t>
+  </si>
+  <si>
+    <t>26/05/22 5:00</t>
+  </si>
+  <si>
+    <t>27/05/22 5:00</t>
+  </si>
+  <si>
+    <t>23/05/22 23:00</t>
+  </si>
+  <si>
+    <t>24/05/22 23:00</t>
+  </si>
+  <si>
+    <t>25/05/22 23:00</t>
+  </si>
+  <si>
+    <t>26/05/22 23:00</t>
+  </si>
+  <si>
+    <t>27/05/22 23:00</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3599,6 +3629,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -3644,7 +3680,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4012,11 +4048,11 @@
       <c r="B2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="2">
-        <v>44704.208333333336</v>
-      </c>
-      <c r="D2" s="2">
-        <v>44704.958333333336</v>
+      <c r="C2" s="2" t="s">
+        <v>1184</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>1189</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -4026,11 +4062,11 @@
       <c r="B3" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="2">
-        <v>44704.208333333336</v>
-      </c>
-      <c r="D3" s="2">
-        <v>44704.958333333336</v>
+      <c r="C3" s="2" t="s">
+        <v>1184</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>1189</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -4040,11 +4076,11 @@
       <c r="B4" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="2">
-        <v>44705.208333333336</v>
-      </c>
-      <c r="D4" s="2">
-        <v>44705.958333333336</v>
+      <c r="C4" s="2" t="s">
+        <v>1185</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>1190</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -4054,11 +4090,11 @@
       <c r="B5" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="2">
-        <v>44705.208333333336</v>
-      </c>
-      <c r="D5" s="2">
-        <v>44705.958333333336</v>
+      <c r="C5" s="2" t="s">
+        <v>1185</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>1190</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -4068,11 +4104,11 @@
       <c r="B6" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="2">
-        <v>44706.208333333336</v>
-      </c>
-      <c r="D6" s="2">
-        <v>44706.958333333336</v>
+      <c r="C6" s="2" t="s">
+        <v>1186</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>1191</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -4082,11 +4118,11 @@
       <c r="B7" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="2">
-        <v>44707.208333333336</v>
-      </c>
-      <c r="D7" s="2">
-        <v>44707.958333333336</v>
+      <c r="C7" s="2" t="s">
+        <v>1187</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>1192</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -4096,11 +4132,11 @@
       <c r="B8" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="2">
-        <v>44707.208333333336</v>
-      </c>
-      <c r="D8" s="2">
-        <v>44707.958333333336</v>
+      <c r="C8" s="2" t="s">
+        <v>1187</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>1192</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -4110,11 +4146,11 @@
       <c r="B9" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="2">
-        <v>44708.208333333336</v>
-      </c>
-      <c r="D9" s="2">
-        <v>44708.958333333336</v>
+      <c r="C9" s="2" t="s">
+        <v>1188</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>1193</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -4124,14 +4160,15 @@
       <c r="B10" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="2">
-        <v>44708.208333333336</v>
-      </c>
-      <c r="D10" s="2">
-        <v>44708.958333333336</v>
+      <c r="C10" s="2" t="s">
+        <v>1188</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>1193</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -4177,6 +4214,9 @@
       <c r="B2">
         <v>166461</v>
       </c>
+      <c r="C2">
+        <v>10</v>
+      </c>
       <c r="D2" t="s">
         <v>1019</v>
       </c>
@@ -4197,6 +4237,9 @@
       <c r="B3">
         <v>166479</v>
       </c>
+      <c r="C3">
+        <v>11</v>
+      </c>
       <c r="D3" t="s">
         <v>1020</v>
       </c>
@@ -4217,6 +4260,9 @@
       <c r="B4">
         <v>166522</v>
       </c>
+      <c r="C4">
+        <v>12</v>
+      </c>
       <c r="D4" t="s">
         <v>1021</v>
       </c>
@@ -4237,6 +4283,9 @@
       <c r="B5">
         <v>166488</v>
       </c>
+      <c r="C5">
+        <v>13</v>
+      </c>
       <c r="D5" t="s">
         <v>1022</v>
       </c>
@@ -4257,6 +4306,9 @@
       <c r="B6">
         <v>166495</v>
       </c>
+      <c r="C6">
+        <v>14</v>
+      </c>
       <c r="D6" t="s">
         <v>1023</v>
       </c>
@@ -4277,6 +4329,9 @@
       <c r="B7">
         <v>166520</v>
       </c>
+      <c r="C7">
+        <v>15</v>
+      </c>
       <c r="D7" t="s">
         <v>1024</v>
       </c>
@@ -4297,6 +4352,9 @@
       <c r="B8">
         <v>166528</v>
       </c>
+      <c r="C8">
+        <v>16</v>
+      </c>
       <c r="D8" t="s">
         <v>1025</v>
       </c>
@@ -4317,6 +4375,9 @@
       <c r="B9">
         <v>166523</v>
       </c>
+      <c r="C9">
+        <v>17</v>
+      </c>
       <c r="D9" t="s">
         <v>1026</v>
       </c>
@@ -4337,6 +4398,9 @@
       <c r="B10">
         <v>166570</v>
       </c>
+      <c r="C10">
+        <v>18</v>
+      </c>
       <c r="D10" t="s">
         <v>1027</v>
       </c>
@@ -4357,6 +4421,9 @@
       <c r="B11">
         <v>166578</v>
       </c>
+      <c r="C11">
+        <v>19</v>
+      </c>
       <c r="D11" t="s">
         <v>1028</v>
       </c>
@@ -4376,6 +4443,9 @@
       </c>
       <c r="B12">
         <v>166569</v>
+      </c>
+      <c r="C12">
+        <v>20</v>
       </c>
       <c r="D12" t="s">
         <v>1029</v>

</xml_diff>

<commit_message>
session with screens and date 2.0
</commit_message>
<xml_diff>
--- a/pm2022/pm2022.xlsx
+++ b/pm2022/pm2022.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/galli/Documents/OrgConferenze/21PisaMeeting/pisameet/pm2022/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC8F2CDB-704C-354C-9E03-A9EE769BD09B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60E86944-7FF7-7A48-B832-75DE85369EB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3583,34 +3583,34 @@
     <t>Jagiellonian University</t>
   </si>
   <si>
-    <t>23/05/22 5:00</t>
-  </si>
-  <si>
-    <t>24/05/22 5:00</t>
-  </si>
-  <si>
-    <t>25/05/22 5:00</t>
-  </si>
-  <si>
-    <t>26/05/22 5:00</t>
-  </si>
-  <si>
-    <t>27/05/22 5:00</t>
-  </si>
-  <si>
-    <t>23/05/22 23:00</t>
-  </si>
-  <si>
-    <t>24/05/22 23:00</t>
-  </si>
-  <si>
-    <t>25/05/22 23:00</t>
-  </si>
-  <si>
-    <t>26/05/22 23:00</t>
-  </si>
-  <si>
-    <t>27/05/22 23:00</t>
+    <t>23/05/2022 5:00</t>
+  </si>
+  <si>
+    <t>24/05/2022 5:00</t>
+  </si>
+  <si>
+    <t>25/05/2022 5:00</t>
+  </si>
+  <si>
+    <t>26/05/2022 5:00</t>
+  </si>
+  <si>
+    <t>27/05/2022 5:00</t>
+  </si>
+  <si>
+    <t>23/05/2022 23:00</t>
+  </si>
+  <si>
+    <t>24/05/2022 23:00</t>
+  </si>
+  <si>
+    <t>25/05/2022 23:00</t>
+  </si>
+  <si>
+    <t>26/05/2022 23:00</t>
+  </si>
+  <si>
+    <t>27/05/2022 23:00</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Techtra -> Wroclaw University of Science and Technology
</commit_message>
<xml_diff>
--- a/pm2022/pm2022.xlsx
+++ b/pm2022/pm2022.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/galli/Documents/OrgConferenze/21PisaMeeting/pisameet/pm2022/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7D78DB9-BC47-4B40-9AFD-F06C462A442E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C38D547-E91A-7544-9F56-D1804DB5D30E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19360" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1501,9 +1501,6 @@
     <t>Paul Scherrer Institut - ETH Zürich</t>
   </si>
   <si>
-    <t>TTA Techtra</t>
-  </si>
-  <si>
     <t>12</t>
   </si>
   <si>
@@ -3620,6 +3617,9 @@
   </si>
   <si>
     <t>Università degli studi dell'Insubria</t>
+  </si>
+  <si>
+    <t>Wroclaw University of Science and Technology</t>
   </si>
 </sst>
 </file>
@@ -4058,10 +4058,10 @@
         <v>13</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>1182</v>
+        <v>1181</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -4072,10 +4072,10 @@
         <v>14</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>1182</v>
+        <v>1181</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -4086,10 +4086,10 @@
         <v>15</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -4100,10 +4100,10 @@
         <v>16</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -4114,10 +4114,10 @@
         <v>17</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -4128,10 +4128,10 @@
         <v>18</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -4142,10 +4142,10 @@
         <v>19</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -4156,10 +4156,10 @@
         <v>20</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -4170,10 +4170,10 @@
         <v>21</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
     </row>
   </sheetData>
@@ -4218,7 +4218,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="B2">
         <v>166461</v>
@@ -4227,21 +4227,21 @@
         <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
       <c r="E2" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
       <c r="F2" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
       <c r="G2" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="B3">
         <v>166479</v>
@@ -4250,21 +4250,21 @@
         <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="E3" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="F3" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
       <c r="G3" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="B4">
         <v>166522</v>
@@ -4273,21 +4273,21 @@
         <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="E4" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
       <c r="F4" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
       <c r="G4" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="B5">
         <v>166488</v>
@@ -4296,21 +4296,21 @@
         <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="E5" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="F5" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="G5" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="B6">
         <v>166495</v>
@@ -4319,13 +4319,13 @@
         <v>14</v>
       </c>
       <c r="D6" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="E6" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="F6" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="G6" t="s">
         <v>118</v>
@@ -4333,7 +4333,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="B7">
         <v>166520</v>
@@ -4342,21 +4342,21 @@
         <v>15</v>
       </c>
       <c r="D7" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
       <c r="E7" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="F7" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="G7" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="B8">
         <v>166528</v>
@@ -4365,13 +4365,13 @@
         <v>16</v>
       </c>
       <c r="D8" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="E8" t="s">
         <v>315</v>
       </c>
       <c r="F8" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="G8" t="s">
         <v>118</v>
@@ -4379,7 +4379,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="B9">
         <v>166523</v>
@@ -4388,21 +4388,21 @@
         <v>17</v>
       </c>
       <c r="D9" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="E9" t="s">
         <v>344</v>
       </c>
       <c r="F9" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="G9" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="B10">
         <v>166570</v>
@@ -4411,13 +4411,13 @@
         <v>18</v>
       </c>
       <c r="D10" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="E10" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="F10" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="G10" t="s">
         <v>118</v>
@@ -4425,7 +4425,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="B11">
         <v>166578</v>
@@ -4434,7 +4434,7 @@
         <v>19</v>
       </c>
       <c r="D11" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="E11" t="s">
         <v>314</v>
@@ -4448,7 +4448,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="B12">
         <v>166569</v>
@@ -4457,21 +4457,21 @@
         <v>20</v>
       </c>
       <c r="D12" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="E12" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="F12" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="G12" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="B13">
         <v>166734</v>
@@ -4480,21 +4480,21 @@
         <v>10</v>
       </c>
       <c r="D13" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="E13" t="s">
         <v>74</v>
       </c>
       <c r="F13" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="G13" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="B14">
         <v>166806</v>
@@ -4503,7 +4503,7 @@
         <v>11</v>
       </c>
       <c r="D14" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="E14" t="s">
         <v>314</v>
@@ -4517,7 +4517,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="B15">
         <v>166637</v>
@@ -4526,13 +4526,13 @@
         <v>12</v>
       </c>
       <c r="D15" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="E15" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="F15" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
       <c r="G15" t="s">
         <v>118</v>
@@ -4540,7 +4540,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="B16">
         <v>166648</v>
@@ -4549,21 +4549,21 @@
         <v>13</v>
       </c>
       <c r="D16" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="E16" t="s">
         <v>343</v>
       </c>
       <c r="F16" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="G16" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="B17">
         <v>166676</v>
@@ -4572,21 +4572,21 @@
         <v>14</v>
       </c>
       <c r="D17" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="E17" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="F17" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="G17" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="B18">
         <v>166715</v>
@@ -4595,21 +4595,21 @@
         <v>15</v>
       </c>
       <c r="D18" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="E18" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
       <c r="F18" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
       <c r="G18" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="B19">
         <v>166692</v>
@@ -4618,13 +4618,13 @@
         <v>16</v>
       </c>
       <c r="D19" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="E19" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="F19" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="G19" t="s">
         <v>118</v>
@@ -4632,7 +4632,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="B20">
         <v>166694</v>
@@ -4641,13 +4641,13 @@
         <v>17</v>
       </c>
       <c r="D20" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="E20" t="s">
         <v>169</v>
       </c>
       <c r="F20" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="G20" t="s">
         <v>118</v>
@@ -4655,7 +4655,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="B21">
         <v>166709</v>
@@ -4664,21 +4664,21 @@
         <v>18</v>
       </c>
       <c r="D21" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="E21" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
       <c r="F21" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="G21" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="B22">
         <v>166717</v>
@@ -4687,21 +4687,21 @@
         <v>19</v>
       </c>
       <c r="D22" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="E22" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="F22" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="G22" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="B23">
         <v>166751</v>
@@ -4710,21 +4710,21 @@
         <v>20</v>
       </c>
       <c r="D23" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="E23" t="s">
         <v>329</v>
       </c>
       <c r="F23" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="G23" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="B24">
         <v>166777</v>
@@ -4733,21 +4733,21 @@
         <v>10</v>
       </c>
       <c r="D24" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
       <c r="E24" t="s">
         <v>321</v>
       </c>
       <c r="F24" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="G24" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="B25">
         <v>166789</v>
@@ -4756,7 +4756,7 @@
         <v>11</v>
       </c>
       <c r="D25" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
       <c r="E25" t="s">
         <v>314</v>
@@ -4770,7 +4770,7 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="B26">
         <v>166791</v>
@@ -4779,21 +4779,21 @@
         <v>12</v>
       </c>
       <c r="D26" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
       <c r="E26" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="F26" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="G26" t="s">
-        <v>1167</v>
+        <v>1166</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="B27">
         <v>166819</v>
@@ -4802,21 +4802,21 @@
         <v>13</v>
       </c>
       <c r="D27" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="E27" t="s">
         <v>84</v>
       </c>
       <c r="F27" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="G27" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="B28">
         <v>166527</v>
@@ -4825,21 +4825,21 @@
         <v>14</v>
       </c>
       <c r="D28" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="E28" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="F28" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="G28" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="B29">
         <v>166610</v>
@@ -4848,21 +4848,21 @@
         <v>15</v>
       </c>
       <c r="D29" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="E29" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
       <c r="F29" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="G29" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="B30">
         <v>166512</v>
@@ -4871,13 +4871,13 @@
         <v>16</v>
       </c>
       <c r="D30" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="E30" t="s">
         <v>329</v>
       </c>
       <c r="F30" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="G30" t="s">
         <v>118</v>
@@ -4885,7 +4885,7 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="B31">
         <v>166526</v>
@@ -4894,13 +4894,13 @@
         <v>17</v>
       </c>
       <c r="D31" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="E31" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="F31" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="G31" t="s">
         <v>118</v>
@@ -4908,7 +4908,7 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="B32">
         <v>166530</v>
@@ -4917,13 +4917,13 @@
         <v>18</v>
       </c>
       <c r="D32" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="E32" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="F32" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="G32" t="s">
         <v>118</v>
@@ -4931,7 +4931,7 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="B33">
         <v>166602</v>
@@ -4940,13 +4940,13 @@
         <v>19</v>
       </c>
       <c r="D33" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="E33" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="F33" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="G33" t="s">
         <v>118</v>
@@ -4954,7 +4954,7 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="B34">
         <v>166605</v>
@@ -4963,13 +4963,13 @@
         <v>20</v>
       </c>
       <c r="D34" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="E34" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="F34" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
       <c r="G34" t="s">
         <v>118</v>
@@ -4977,7 +4977,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="B35">
         <v>166614</v>
@@ -4986,21 +4986,21 @@
         <v>10</v>
       </c>
       <c r="D35" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="E35" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
       <c r="F35" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
       <c r="G35" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="B36">
         <v>166618</v>
@@ -5009,13 +5009,13 @@
         <v>11</v>
       </c>
       <c r="D36" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="E36" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="F36" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="G36" t="s">
         <v>118</v>
@@ -5023,7 +5023,7 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="B37">
         <v>166620</v>
@@ -5032,21 +5032,21 @@
         <v>12</v>
       </c>
       <c r="D37" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="E37" t="s">
         <v>174</v>
       </c>
       <c r="F37" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="G37" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="B38">
         <v>166621</v>
@@ -5055,21 +5055,21 @@
         <v>13</v>
       </c>
       <c r="D38" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="E38" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="F38" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="G38" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="B39">
         <v>166632</v>
@@ -5078,21 +5078,21 @@
         <v>14</v>
       </c>
       <c r="D39" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="E39" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
       <c r="F39" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
       <c r="G39" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="B40">
         <v>166649</v>
@@ -5101,13 +5101,13 @@
         <v>15</v>
       </c>
       <c r="D40" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="E40" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="F40" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="G40" t="s">
         <v>118</v>
@@ -5115,7 +5115,7 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="B41">
         <v>166652</v>
@@ -5124,13 +5124,13 @@
         <v>16</v>
       </c>
       <c r="D41" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="E41" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
       <c r="F41" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="G41" t="s">
         <v>118</v>
@@ -5138,7 +5138,7 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="B42">
         <v>166672</v>
@@ -5147,21 +5147,21 @@
         <v>17</v>
       </c>
       <c r="D42" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="E42" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
       <c r="F42" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
       <c r="G42" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="B43">
         <v>166677</v>
@@ -5170,21 +5170,21 @@
         <v>18</v>
       </c>
       <c r="D43" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="E43" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="F43" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="G43" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="B44">
         <v>166680</v>
@@ -5193,13 +5193,13 @@
         <v>19</v>
       </c>
       <c r="D44" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="E44" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
       <c r="F44" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="G44" t="s">
         <v>484</v>
@@ -5207,7 +5207,7 @@
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="B45">
         <v>166718</v>
@@ -5216,21 +5216,21 @@
         <v>20</v>
       </c>
       <c r="D45" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="E45" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="F45" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="G45" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="B46">
         <v>166720</v>
@@ -5239,7 +5239,7 @@
         <v>10</v>
       </c>
       <c r="D46" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="E46" t="s">
         <v>314</v>
@@ -5253,7 +5253,7 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="B47">
         <v>166742</v>
@@ -5262,13 +5262,13 @@
         <v>11</v>
       </c>
       <c r="D47" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="E47" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="F47" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="G47" t="s">
         <v>118</v>
@@ -5276,7 +5276,7 @@
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="B48">
         <v>166752</v>
@@ -5285,13 +5285,13 @@
         <v>12</v>
       </c>
       <c r="D48" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="E48" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="F48" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="G48" t="s">
         <v>118</v>
@@ -5299,7 +5299,7 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="B49">
         <v>166761</v>
@@ -5308,21 +5308,21 @@
         <v>13</v>
       </c>
       <c r="D49" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="E49" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
       <c r="F49" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="G49" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="B50">
         <v>166772</v>
@@ -5331,21 +5331,21 @@
         <v>14</v>
       </c>
       <c r="D50" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="E50" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
       <c r="F50" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="G50" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="B51">
         <v>166786</v>
@@ -5354,13 +5354,13 @@
         <v>15</v>
       </c>
       <c r="D51" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="E51" t="s">
         <v>321</v>
       </c>
       <c r="F51" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="G51" t="s">
         <v>118</v>
@@ -5368,7 +5368,7 @@
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="B52">
         <v>166815</v>
@@ -5377,21 +5377,21 @@
         <v>16</v>
       </c>
       <c r="D52" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="E52" t="s">
         <v>309</v>
       </c>
       <c r="F52" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="G52" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="B53">
         <v>166816</v>
@@ -5400,13 +5400,13 @@
         <v>17</v>
       </c>
       <c r="D53" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="E53" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="F53" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="G53" t="s">
         <v>118</v>
@@ -5414,7 +5414,7 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="B54">
         <v>166817</v>
@@ -5423,13 +5423,13 @@
         <v>18</v>
       </c>
       <c r="D54" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="E54" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="F54" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="G54" t="s">
         <v>118</v>
@@ -5437,7 +5437,7 @@
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="B55">
         <v>167826</v>
@@ -5446,21 +5446,21 @@
         <v>19</v>
       </c>
       <c r="D55" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="E55" t="s">
-        <v>1101</v>
+        <v>1100</v>
       </c>
       <c r="F55" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="G55" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="B56">
         <v>167837</v>
@@ -5469,21 +5469,21 @@
         <v>20</v>
       </c>
       <c r="D56" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="E56" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
       <c r="F56" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="G56" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="B57">
         <v>170164</v>
@@ -5492,13 +5492,13 @@
         <v>10</v>
       </c>
       <c r="D57" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
       <c r="E57" t="s">
         <v>344</v>
       </c>
       <c r="F57" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="G57" t="s">
         <v>118</v>
@@ -5506,7 +5506,7 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="B58">
         <v>170518</v>
@@ -5515,16 +5515,16 @@
         <v>11</v>
       </c>
       <c r="D58" t="s">
-        <v>1073</v>
+        <v>1072</v>
       </c>
       <c r="E58" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="F58" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="G58" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
     </row>
   </sheetData>
@@ -7199,10 +7199,10 @@
         <v>286</v>
       </c>
       <c r="E30" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="F30" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
       <c r="G30" t="s">
         <v>403</v>
@@ -8118,7 +8118,7 @@
         <v>482</v>
       </c>
       <c r="G21" t="s">
-        <v>490</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -8132,16 +8132,16 @@
         <v>17</v>
       </c>
       <c r="D22" t="s">
+        <v>1192</v>
+      </c>
+      <c r="E22" t="s">
         <v>1193</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>1194</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>1195</v>
-      </c>
-      <c r="G22" t="s">
-        <v>1196</v>
       </c>
     </row>
   </sheetData>
@@ -8185,7 +8185,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="B2">
         <v>166466</v>
@@ -8194,21 +8194,21 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="E2" t="s">
         <v>164</v>
       </c>
       <c r="F2" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="G2" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B3">
         <v>166467</v>
@@ -8217,21 +8217,21 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="E3" t="s">
         <v>74</v>
       </c>
       <c r="F3" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="G3" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B4">
         <v>166519</v>
@@ -8240,13 +8240,13 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="E4" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="F4" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="G4" t="s">
         <v>118</v>
@@ -8254,7 +8254,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B5">
         <v>166550</v>
@@ -8263,21 +8263,21 @@
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="E5" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="F5" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="G5" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B6">
         <v>166645</v>
@@ -8286,21 +8286,21 @@
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="E6" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="F6" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G6" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B7">
         <v>166643</v>
@@ -8309,21 +8309,21 @@
         <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="E7" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="F7" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="G7" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B8">
         <v>166685</v>
@@ -8332,21 +8332,21 @@
         <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="E8" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="F8" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="G8" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B9">
         <v>166810</v>
@@ -8355,21 +8355,21 @@
         <v>8</v>
       </c>
       <c r="D9" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="E9" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="F9" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="G9" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B10">
         <v>166740</v>
@@ -8378,7 +8378,7 @@
         <v>9</v>
       </c>
       <c r="D10" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="E10" t="s">
         <v>177</v>
@@ -8387,12 +8387,12 @@
         <v>195</v>
       </c>
       <c r="G10" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="B11">
         <v>166754</v>
@@ -8401,13 +8401,13 @@
         <v>10</v>
       </c>
       <c r="D11" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="E11" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="F11" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="G11" t="s">
         <v>118</v>
@@ -8415,7 +8415,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B12">
         <v>166775</v>
@@ -8424,13 +8424,13 @@
         <v>11</v>
       </c>
       <c r="D12" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E12" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="F12" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="G12" t="s">
         <v>118</v>
@@ -8438,7 +8438,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B13">
         <v>166475</v>
@@ -8447,21 +8447,21 @@
         <v>12</v>
       </c>
       <c r="D13" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="E13" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="F13" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="G13" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B14">
         <v>166511</v>
@@ -8470,21 +8470,21 @@
         <v>13</v>
       </c>
       <c r="D14" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="E14" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="F14" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="G14" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B15">
         <v>166518</v>
@@ -8493,13 +8493,13 @@
         <v>14</v>
       </c>
       <c r="D15" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="E15" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="F15" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="G15" t="s">
         <v>118</v>
@@ -8507,7 +8507,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B16">
         <v>166524</v>
@@ -8516,21 +8516,21 @@
         <v>15</v>
       </c>
       <c r="D16" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="E16" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="F16" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="G16" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B17">
         <v>166525</v>
@@ -8539,13 +8539,13 @@
         <v>16</v>
       </c>
       <c r="D17" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="E17" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="F17" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="G17" t="s">
         <v>118</v>
@@ -8553,7 +8553,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="B18">
         <v>166563</v>
@@ -8562,13 +8562,13 @@
         <v>17</v>
       </c>
       <c r="D18" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="E18" t="s">
         <v>455</v>
       </c>
       <c r="F18" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="G18" t="s">
         <v>114</v>
@@ -8576,7 +8576,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B19">
         <v>166608</v>
@@ -8585,21 +8585,21 @@
         <v>18</v>
       </c>
       <c r="D19" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="E19" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="F19" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="G19" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="B20">
         <v>166659</v>
@@ -8608,21 +8608,21 @@
         <v>19</v>
       </c>
       <c r="D20" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="E20" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="F20" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="G20" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="B21">
         <v>166664</v>
@@ -8631,13 +8631,13 @@
         <v>20</v>
       </c>
       <c r="D21" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="E21" t="s">
         <v>315</v>
       </c>
       <c r="F21" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="G21" t="s">
         <v>118</v>
@@ -8645,7 +8645,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B22">
         <v>166727</v>
@@ -8654,21 +8654,21 @@
         <v>1</v>
       </c>
       <c r="D22" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="E22" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="F22" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="G22" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="B23">
         <v>166738</v>
@@ -8677,13 +8677,13 @@
         <v>2</v>
       </c>
       <c r="D23" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="E23" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="F23" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="G23" t="s">
         <v>118</v>
@@ -8730,7 +8730,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="B2">
         <v>166656</v>
@@ -8739,13 +8739,13 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="E2" t="s">
         <v>174</v>
       </c>
       <c r="F2" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="G2" t="s">
         <v>118</v>
@@ -8753,7 +8753,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B3">
         <v>166795</v>
@@ -8762,21 +8762,21 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="E3" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="F3" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="G3" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B4">
         <v>166674</v>
@@ -8785,13 +8785,13 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="E4" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="F4" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="G4" t="s">
         <v>118</v>
@@ -8799,7 +8799,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B5">
         <v>166582</v>
@@ -8808,21 +8808,21 @@
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="E5" t="s">
         <v>174</v>
       </c>
       <c r="F5" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="G5" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="B6">
         <v>166679</v>
@@ -8831,21 +8831,21 @@
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="E6" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="F6" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="G6" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B7">
         <v>166794</v>
@@ -8854,21 +8854,21 @@
         <v>2</v>
       </c>
       <c r="D7" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="E7" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="F7" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="G7" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="B8">
         <v>167882</v>
@@ -8877,13 +8877,13 @@
         <v>3</v>
       </c>
       <c r="D8" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="E8" t="s">
         <v>169</v>
       </c>
       <c r="F8" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="G8" t="s">
         <v>118</v>
@@ -8891,7 +8891,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B9">
         <v>166696</v>
@@ -8900,21 +8900,21 @@
         <v>4</v>
       </c>
       <c r="D9" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="E9" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="F9" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="G9" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B10">
         <v>166700</v>
@@ -8923,21 +8923,21 @@
         <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="E10" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="F10" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="G10" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B11">
         <v>166792</v>
@@ -8946,13 +8946,13 @@
         <v>2</v>
       </c>
       <c r="D11" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="E11" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F11" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="G11" t="s">
         <v>118</v>
@@ -8999,7 +8999,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="B2">
         <v>166462</v>
@@ -9008,13 +9008,13 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="E2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F2" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="G2" t="s">
         <v>118</v>
@@ -9022,7 +9022,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B3">
         <v>166486</v>
@@ -9031,21 +9031,21 @@
         <v>6</v>
       </c>
       <c r="D3" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="E3" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="F3" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="G3" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B4">
         <v>166545</v>
@@ -9054,13 +9054,13 @@
         <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="E4" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="F4" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="G4" t="s">
         <v>118</v>
@@ -9068,7 +9068,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="B5">
         <v>166557</v>
@@ -9077,21 +9077,21 @@
         <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="E5" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="F5" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="G5" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B6">
         <v>166566</v>
@@ -9100,13 +9100,13 @@
         <v>9</v>
       </c>
       <c r="D6" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="E6" t="s">
         <v>174</v>
       </c>
       <c r="F6" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="G6" t="s">
         <v>118</v>
@@ -9114,7 +9114,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B7">
         <v>166600</v>
@@ -9123,13 +9123,13 @@
         <v>10</v>
       </c>
       <c r="D7" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="E7" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="F7" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="G7" t="s">
         <v>118</v>
@@ -9137,7 +9137,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="B8">
         <v>166603</v>
@@ -9146,13 +9146,13 @@
         <v>11</v>
       </c>
       <c r="D8" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="E8" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="F8" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="G8" t="s">
         <v>118</v>
@@ -9160,7 +9160,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B9">
         <v>166624</v>
@@ -9169,13 +9169,13 @@
         <v>12</v>
       </c>
       <c r="D9" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="E9" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="F9" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="G9" t="s">
         <v>486</v>
@@ -9183,7 +9183,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="B10">
         <v>166628</v>
@@ -9192,13 +9192,13 @@
         <v>13</v>
       </c>
       <c r="D10" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="E10" t="s">
         <v>169</v>
       </c>
       <c r="F10" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="G10" t="s">
         <v>118</v>
@@ -9206,7 +9206,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="B11">
         <v>166636</v>
@@ -9215,13 +9215,13 @@
         <v>14</v>
       </c>
       <c r="D11" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="E11" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="F11" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="G11" t="s">
         <v>118</v>
@@ -9229,7 +9229,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="B12">
         <v>166640</v>
@@ -9238,21 +9238,21 @@
         <v>15</v>
       </c>
       <c r="D12" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="E12" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="F12" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="G12" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="B13">
         <v>166668</v>
@@ -9261,13 +9261,13 @@
         <v>16</v>
       </c>
       <c r="D13" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E13" t="s">
         <v>461</v>
       </c>
       <c r="F13" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="G13" t="s">
         <v>118</v>
@@ -9275,7 +9275,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B14">
         <v>166682</v>
@@ -9284,13 +9284,13 @@
         <v>17</v>
       </c>
       <c r="D14" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E14" t="s">
         <v>88</v>
       </c>
       <c r="F14" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="G14" t="s">
         <v>118</v>
@@ -9298,7 +9298,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B15">
         <v>166705</v>
@@ -9307,13 +9307,13 @@
         <v>18</v>
       </c>
       <c r="D15" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="E15" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="F15" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="G15" t="s">
         <v>118</v>
@@ -9321,7 +9321,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B16">
         <v>166716</v>
@@ -9330,21 +9330,21 @@
         <v>19</v>
       </c>
       <c r="D16" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="E16" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="F16" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="G16" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B17">
         <v>166743</v>
@@ -9353,13 +9353,13 @@
         <v>20</v>
       </c>
       <c r="D17" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="E17" t="s">
         <v>169</v>
       </c>
       <c r="F17" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="G17" t="s">
         <v>118</v>
@@ -9367,7 +9367,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B18">
         <v>166814</v>
@@ -9376,13 +9376,13 @@
         <v>5</v>
       </c>
       <c r="D18" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E18" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="F18" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="G18" t="s">
         <v>121</v>
@@ -9390,7 +9390,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B19">
         <v>166497</v>
@@ -9399,13 +9399,13 @@
         <v>6</v>
       </c>
       <c r="D19" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E19" t="s">
         <v>167</v>
       </c>
       <c r="F19" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="G19" t="s">
         <v>118</v>
@@ -9413,7 +9413,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="B20">
         <v>166733</v>
@@ -9422,13 +9422,13 @@
         <v>7</v>
       </c>
       <c r="D20" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="E20" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="F20" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="G20" t="s">
         <v>118</v>
@@ -9436,7 +9436,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B21">
         <v>166496</v>
@@ -9445,13 +9445,13 @@
         <v>8</v>
       </c>
       <c r="D21" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="E21" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="F21" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="G21" t="s">
         <v>118</v>
@@ -9459,7 +9459,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B22">
         <v>166783</v>
@@ -9468,13 +9468,13 @@
         <v>9</v>
       </c>
       <c r="D22" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="E22" t="s">
         <v>85</v>
       </c>
       <c r="F22" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="G22" t="s">
         <v>118</v>
@@ -9482,7 +9482,7 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="B23">
         <v>166468</v>
@@ -9491,13 +9491,13 @@
         <v>10</v>
       </c>
       <c r="D23" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="E23" t="s">
         <v>164</v>
       </c>
       <c r="F23" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="G23" t="s">
         <v>118</v>
@@ -9505,7 +9505,7 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="B24">
         <v>166494</v>
@@ -9514,21 +9514,21 @@
         <v>11</v>
       </c>
       <c r="D24" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="E24" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="F24" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="G24" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B25">
         <v>166509</v>
@@ -9537,21 +9537,21 @@
         <v>12</v>
       </c>
       <c r="D25" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="E25" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="F25" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G25" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="B26">
         <v>166531</v>
@@ -9560,21 +9560,21 @@
         <v>13</v>
       </c>
       <c r="D26" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E26" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="F26" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="G26" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B27">
         <v>166532</v>
@@ -9583,13 +9583,13 @@
         <v>14</v>
       </c>
       <c r="D27" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="E27" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="F27" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="G27" t="s">
         <v>118</v>
@@ -9597,7 +9597,7 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="B28">
         <v>166559</v>
@@ -9606,21 +9606,21 @@
         <v>15</v>
       </c>
       <c r="D28" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="E28" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="F28" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="G28" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B29">
         <v>166564</v>
@@ -9629,13 +9629,13 @@
         <v>16</v>
       </c>
       <c r="D29" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="E29" t="s">
         <v>169</v>
       </c>
       <c r="F29" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="G29" t="s">
         <v>118</v>
@@ -9643,7 +9643,7 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="B30">
         <v>166565</v>
@@ -9652,21 +9652,21 @@
         <v>17</v>
       </c>
       <c r="D30" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="E30" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="F30" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="G30" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B31">
         <v>166606</v>
@@ -9675,13 +9675,13 @@
         <v>18</v>
       </c>
       <c r="D31" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="E31" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="F31" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="G31" t="s">
         <v>118</v>
@@ -9689,7 +9689,7 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B32">
         <v>166658</v>
@@ -9698,13 +9698,13 @@
         <v>19</v>
       </c>
       <c r="D32" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="E32" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="F32" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="G32" t="s">
         <v>406</v>
@@ -9712,7 +9712,7 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="B33">
         <v>166667</v>
@@ -9721,13 +9721,13 @@
         <v>20</v>
       </c>
       <c r="D33" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="E33" t="s">
         <v>169</v>
       </c>
       <c r="F33" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="G33" t="s">
         <v>118</v>
@@ -9735,7 +9735,7 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B34">
         <v>166671</v>
@@ -9744,13 +9744,13 @@
         <v>5</v>
       </c>
       <c r="D34" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="E34" t="s">
         <v>169</v>
       </c>
       <c r="F34" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="G34" t="s">
         <v>118</v>
@@ -9758,7 +9758,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B35">
         <v>166684</v>
@@ -9767,21 +9767,21 @@
         <v>6</v>
       </c>
       <c r="D35" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="E35" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="F35" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="G35" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B36">
         <v>166730</v>
@@ -9790,13 +9790,13 @@
         <v>7</v>
       </c>
       <c r="D36" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="E36" t="s">
         <v>321</v>
       </c>
       <c r="F36" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="G36" t="s">
         <v>118</v>
@@ -9804,7 +9804,7 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B37">
         <v>166736</v>
@@ -9813,13 +9813,13 @@
         <v>8</v>
       </c>
       <c r="D37" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="E37" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="F37" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="G37" t="s">
         <v>118</v>
@@ -9827,7 +9827,7 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="B38">
         <v>166739</v>
@@ -9836,21 +9836,21 @@
         <v>9</v>
       </c>
       <c r="D38" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="E38" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="F38" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="G38" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B39">
         <v>166749</v>
@@ -9859,21 +9859,21 @@
         <v>10</v>
       </c>
       <c r="D39" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="E39" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="F39" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="G39" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="B40">
         <v>166766</v>
@@ -9882,13 +9882,13 @@
         <v>11</v>
       </c>
       <c r="D40" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="E40" t="s">
         <v>88</v>
       </c>
       <c r="F40" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="G40" t="s">
         <v>118</v>
@@ -9896,7 +9896,7 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="B41">
         <v>167683</v>
@@ -9905,7 +9905,7 @@
         <v>12</v>
       </c>
       <c r="D41" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="E41" t="s">
         <v>166</v>
@@ -9914,12 +9914,12 @@
         <v>184</v>
       </c>
       <c r="G41" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="B42">
         <v>167825</v>
@@ -9928,16 +9928,16 @@
         <v>13</v>
       </c>
       <c r="D42" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="E42" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="F42" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="G42" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
@@ -10004,7 +10004,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="B2">
         <v>166521</v>
@@ -10013,13 +10013,13 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="E2" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="F2" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="G2" t="s">
         <v>118</v>
@@ -10027,7 +10027,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="B3">
         <v>166516</v>
@@ -10036,21 +10036,21 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="E3" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="F3" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="G3" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="B4">
         <v>166508</v>
@@ -10059,13 +10059,13 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="E4" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="F4" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="G4" t="s">
         <v>118</v>
@@ -10073,7 +10073,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="B5">
         <v>166540</v>
@@ -10082,21 +10082,21 @@
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="E5" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="F5" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="G5" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="B6">
         <v>166541</v>
@@ -10105,21 +10105,21 @@
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="E6" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="F6" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="G6" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="B7">
         <v>166561</v>
@@ -10128,21 +10128,21 @@
         <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="E7" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="F7" t="s">
         <v>371</v>
       </c>
       <c r="G7" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="B8">
         <v>166619</v>
@@ -10151,21 +10151,21 @@
         <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E8" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="F8" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="G8" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="B9">
         <v>166623</v>
@@ -10174,13 +10174,13 @@
         <v>8</v>
       </c>
       <c r="D9" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="E9" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="F9" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="G9" t="s">
         <v>118</v>
@@ -10188,7 +10188,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="B10">
         <v>166630</v>
@@ -10197,13 +10197,13 @@
         <v>9</v>
       </c>
       <c r="D10" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="E10" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="F10" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="G10" t="s">
         <v>118</v>
@@ -10211,7 +10211,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="B11">
         <v>166663</v>
@@ -10220,21 +10220,21 @@
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="E11" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="F11" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="G11" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="B12">
         <v>166673</v>
@@ -10243,21 +10243,21 @@
         <v>2</v>
       </c>
       <c r="D12" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="E12" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="F12" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="G12" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="B13">
         <v>166675</v>
@@ -10266,21 +10266,21 @@
         <v>3</v>
       </c>
       <c r="D13" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="E13" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="F13" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="G13" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="B14">
         <v>166710</v>
@@ -10289,7 +10289,7 @@
         <v>4</v>
       </c>
       <c r="D14" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="E14" t="s">
         <v>314</v>
@@ -10303,7 +10303,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="B15">
         <v>166711</v>
@@ -10312,21 +10312,21 @@
         <v>5</v>
       </c>
       <c r="D15" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="E15" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="F15" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="G15" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="B16">
         <v>166755</v>
@@ -10335,13 +10335,13 @@
         <v>6</v>
       </c>
       <c r="D16" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="E16" t="s">
         <v>174</v>
       </c>
       <c r="F16" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="G16" t="s">
         <v>118</v>
@@ -10349,7 +10349,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="B17">
         <v>166757</v>
@@ -10358,21 +10358,21 @@
         <v>7</v>
       </c>
       <c r="D17" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="E17" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="F17" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="G17" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="B18">
         <v>167481</v>
@@ -10381,13 +10381,13 @@
         <v>8</v>
       </c>
       <c r="D18" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="E18" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="F18" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="G18" t="s">
         <v>114</v>
@@ -10395,7 +10395,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="B19">
         <v>167793</v>
@@ -10404,13 +10404,13 @@
         <v>9</v>
       </c>
       <c r="D19" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="E19" t="s">
         <v>164</v>
       </c>
       <c r="F19" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="G19" t="s">
         <v>118</v>
@@ -10418,7 +10418,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="B20">
         <v>168287</v>
@@ -10427,21 +10427,21 @@
         <v>1</v>
       </c>
       <c r="D20" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="E20" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="F20" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="G20" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="B21">
         <v>166567</v>
@@ -10450,21 +10450,21 @@
         <v>2</v>
       </c>
       <c r="D21" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="E21" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="F21" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="G21" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="B22">
         <v>166538</v>
@@ -10473,21 +10473,21 @@
         <v>3</v>
       </c>
       <c r="D22" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="E22" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="F22" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="G22" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="B23">
         <v>166678</v>
@@ -10496,21 +10496,21 @@
         <v>4</v>
       </c>
       <c r="D23" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="E23" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="F23" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="G23" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="B24">
         <v>167682</v>
@@ -10519,21 +10519,21 @@
         <v>5</v>
       </c>
       <c r="D24" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="E24" t="s">
         <v>343</v>
       </c>
       <c r="F24" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="G24" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="B25">
         <v>166529</v>
@@ -10542,21 +10542,21 @@
         <v>6</v>
       </c>
       <c r="D25" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="E25" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="F25" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="G25" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="B26">
         <v>166472</v>
@@ -10565,21 +10565,21 @@
         <v>7</v>
       </c>
       <c r="D26" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="E26" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="F26" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="G26" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="B27">
         <v>166571</v>
@@ -10588,21 +10588,21 @@
         <v>8</v>
       </c>
       <c r="D27" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="E27" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="F27" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="G27" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B28">
         <v>166575</v>
@@ -10611,13 +10611,13 @@
         <v>9</v>
       </c>
       <c r="D28" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="E28" t="s">
         <v>461</v>
       </c>
       <c r="F28" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="G28" t="s">
         <v>118</v>
@@ -10625,7 +10625,7 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="B29">
         <v>166590</v>
@@ -10634,21 +10634,21 @@
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="E29" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="F29" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="G29" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="B30">
         <v>166598</v>
@@ -10657,21 +10657,21 @@
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="E30" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="F30" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="G30" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="B31">
         <v>166629</v>
@@ -10680,13 +10680,13 @@
         <v>3</v>
       </c>
       <c r="D31" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="E31" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="F31" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="G31" t="s">
         <v>118</v>
@@ -10694,7 +10694,7 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="B32">
         <v>166650</v>
@@ -10703,21 +10703,21 @@
         <v>4</v>
       </c>
       <c r="D32" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="E32" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="F32" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="G32" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="B33">
         <v>166657</v>
@@ -10726,13 +10726,13 @@
         <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="E33" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="F33" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="G33" t="s">
         <v>114</v>
@@ -10740,7 +10740,7 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="B34">
         <v>166687</v>
@@ -10749,21 +10749,21 @@
         <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="E34" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="F34" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="G34" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="B35">
         <v>166691</v>
@@ -10772,7 +10772,7 @@
         <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="E35" t="s">
         <v>339</v>
@@ -10786,7 +10786,7 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="B36">
         <v>166708</v>
@@ -10795,13 +10795,13 @@
         <v>8</v>
       </c>
       <c r="D36" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="E36" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="F36" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="G36" t="s">
         <v>118</v>
@@ -10809,7 +10809,7 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="B37">
         <v>166719</v>
@@ -10818,21 +10818,21 @@
         <v>9</v>
       </c>
       <c r="D37" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="E37" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="F37" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="G37" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="B38">
         <v>166744</v>
@@ -10841,13 +10841,13 @@
         <v>1</v>
       </c>
       <c r="D38" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="E38" t="s">
         <v>325</v>
       </c>
       <c r="F38" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="G38" t="s">
         <v>118</v>
@@ -10855,7 +10855,7 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B39">
         <v>166746</v>
@@ -10864,21 +10864,21 @@
         <v>2</v>
       </c>
       <c r="D39" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="E39" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="F39" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="G39" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="B40">
         <v>166753</v>
@@ -10887,21 +10887,21 @@
         <v>3</v>
       </c>
       <c r="D40" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="E40" t="s">
         <v>315</v>
       </c>
       <c r="F40" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="G40" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B41">
         <v>166779</v>
@@ -10910,13 +10910,13 @@
         <v>4</v>
       </c>
       <c r="D41" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="E41" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="F41" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="G41" t="s">
         <v>118</v>
@@ -10924,7 +10924,7 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="B42">
         <v>166818</v>
@@ -10933,21 +10933,21 @@
         <v>5</v>
       </c>
       <c r="D42" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="E42" t="s">
         <v>84</v>
       </c>
       <c r="F42" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="G42" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="B43">
         <v>167482</v>
@@ -10956,13 +10956,13 @@
         <v>6</v>
       </c>
       <c r="D43" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="E43" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="F43" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="G43" t="s">
         <v>118</v>
@@ -10970,7 +10970,7 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="B44">
         <v>167812</v>
@@ -10979,13 +10979,13 @@
         <v>7</v>
       </c>
       <c r="D44" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="E44" t="s">
         <v>329</v>
       </c>
       <c r="F44" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="G44" t="s">
         <v>118</v>
@@ -10993,7 +10993,7 @@
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="B45">
         <v>171332</v>
@@ -11002,16 +11002,16 @@
         <v>8</v>
       </c>
       <c r="D45" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="E45" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="F45" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="G45" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Program updated, added 184 and remover 423
</commit_message>
<xml_diff>
--- a/pm2022/pm2022.xlsx
+++ b/pm2022/pm2022.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/galli/Documents/OrgConferenze/21PisaMeeting/pisameet/pm2022/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82872C31-8345-6849-A36D-D8732F57186B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1F9749A-8B12-3543-A1FB-EC5559C257D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19360" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19360" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Program" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1506" uniqueCount="1193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1505" uniqueCount="1190">
   <si>
     <t>Session ID</t>
   </si>
@@ -1792,9 +1792,6 @@
     <t>272</t>
   </si>
   <si>
-    <t>423</t>
-  </si>
-  <si>
     <t>204</t>
   </si>
   <si>
@@ -1822,9 +1819,6 @@
     <t>Background of X-ray TES micro-calorimeter arrays for elusive particle experiments</t>
   </si>
   <si>
-    <t>Response characterization of PVT scintillators to alpha and beta/gamma sources for low temperature applications</t>
-  </si>
-  <si>
     <t>Design and preliminary characterizations of traveling wave parametric amplifiers for DARTWARS</t>
   </si>
   <si>
@@ -1873,9 +1867,6 @@
     <t>Vaccaro</t>
   </si>
   <si>
-    <t>Gironi</t>
-  </si>
-  <si>
     <t>Borghesi</t>
   </si>
   <si>
@@ -1897,9 +1888,6 @@
     <t>SRON Leiden</t>
   </si>
   <si>
-    <t>University Milano Bicocca</t>
-  </si>
-  <si>
     <t>GE</t>
   </si>
   <si>
@@ -3608,6 +3596,9 @@
   </si>
   <si>
     <t>The DAQ and clock distribution system of CMS MIP Timing Detector</t>
+  </si>
+  <si>
+    <t>Operational results with the pixelated timing Counter (pTC) of the MEGII experiment during the first year of physics data taking</t>
   </si>
 </sst>
 </file>
@@ -4046,10 +4037,10 @@
         <v>13</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>1169</v>
+        <v>1165</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>1174</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -4060,10 +4051,10 @@
         <v>14</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>1169</v>
+        <v>1165</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>1174</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -4074,10 +4065,10 @@
         <v>15</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1170</v>
+        <v>1166</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>1175</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -4088,10 +4079,10 @@
         <v>16</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>1170</v>
+        <v>1166</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>1175</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -4102,10 +4093,10 @@
         <v>17</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1171</v>
+        <v>1167</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>1176</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -4116,10 +4107,10 @@
         <v>18</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>1172</v>
+        <v>1168</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>1177</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -4130,10 +4121,10 @@
         <v>19</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>1172</v>
+        <v>1168</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>1177</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -4144,10 +4135,10 @@
         <v>20</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>1173</v>
+        <v>1169</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>1178</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -4158,10 +4149,10 @@
         <v>21</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>1173</v>
+        <v>1169</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>1178</v>
+        <v>1174</v>
       </c>
     </row>
   </sheetData>
@@ -4206,7 +4197,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>950</v>
+        <v>946</v>
       </c>
       <c r="B2">
         <v>166461</v>
@@ -4215,21 +4206,21 @@
         <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>1007</v>
+        <v>1003</v>
       </c>
       <c r="E2" t="s">
-        <v>1064</v>
+        <v>1060</v>
       </c>
       <c r="F2" t="s">
-        <v>1092</v>
+        <v>1088</v>
       </c>
       <c r="G2" t="s">
-        <v>1140</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>951</v>
+        <v>947</v>
       </c>
       <c r="B3">
         <v>166479</v>
@@ -4238,21 +4229,21 @@
         <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>1008</v>
+        <v>1004</v>
       </c>
       <c r="E3" t="s">
-        <v>1065</v>
+        <v>1061</v>
       </c>
       <c r="F3" t="s">
-        <v>1093</v>
+        <v>1089</v>
       </c>
       <c r="G3" t="s">
-        <v>1141</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>952</v>
+        <v>948</v>
       </c>
       <c r="B4">
         <v>166522</v>
@@ -4261,21 +4252,21 @@
         <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>1009</v>
+        <v>1005</v>
       </c>
       <c r="E4" t="s">
-        <v>1066</v>
+        <v>1062</v>
       </c>
       <c r="F4" t="s">
-        <v>1094</v>
+        <v>1090</v>
       </c>
       <c r="G4" t="s">
-        <v>1142</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>953</v>
+        <v>949</v>
       </c>
       <c r="B5">
         <v>166488</v>
@@ -4284,21 +4275,21 @@
         <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>1010</v>
+        <v>1006</v>
       </c>
       <c r="E5" t="s">
-        <v>1067</v>
+        <v>1063</v>
       </c>
       <c r="F5" t="s">
-        <v>1095</v>
+        <v>1091</v>
       </c>
       <c r="G5" t="s">
-        <v>1143</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>954</v>
+        <v>950</v>
       </c>
       <c r="B6">
         <v>166495</v>
@@ -4307,13 +4298,13 @@
         <v>14</v>
       </c>
       <c r="D6" t="s">
-        <v>1011</v>
+        <v>1007</v>
       </c>
       <c r="E6" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="F6" t="s">
-        <v>1096</v>
+        <v>1092</v>
       </c>
       <c r="G6" t="s">
         <v>118</v>
@@ -4321,7 +4312,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>955</v>
+        <v>951</v>
       </c>
       <c r="B7">
         <v>166520</v>
@@ -4330,21 +4321,21 @@
         <v>15</v>
       </c>
       <c r="D7" t="s">
-        <v>1012</v>
+        <v>1008</v>
       </c>
       <c r="E7" t="s">
-        <v>874</v>
+        <v>870</v>
       </c>
       <c r="F7" t="s">
-        <v>1097</v>
+        <v>1093</v>
       </c>
       <c r="G7" t="s">
-        <v>1144</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>956</v>
+        <v>952</v>
       </c>
       <c r="B8">
         <v>166528</v>
@@ -4353,13 +4344,13 @@
         <v>16</v>
       </c>
       <c r="D8" t="s">
-        <v>1013</v>
+        <v>1009</v>
       </c>
       <c r="E8" t="s">
         <v>312</v>
       </c>
       <c r="F8" t="s">
-        <v>1098</v>
+        <v>1094</v>
       </c>
       <c r="G8" t="s">
         <v>118</v>
@@ -4367,7 +4358,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>957</v>
+        <v>953</v>
       </c>
       <c r="B9">
         <v>166523</v>
@@ -4376,21 +4367,21 @@
         <v>17</v>
       </c>
       <c r="D9" t="s">
-        <v>1014</v>
+        <v>1010</v>
       </c>
       <c r="E9" t="s">
         <v>341</v>
       </c>
       <c r="F9" t="s">
-        <v>1099</v>
+        <v>1095</v>
       </c>
       <c r="G9" t="s">
-        <v>1145</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>958</v>
+        <v>954</v>
       </c>
       <c r="B10">
         <v>166570</v>
@@ -4399,13 +4390,13 @@
         <v>18</v>
       </c>
       <c r="D10" t="s">
-        <v>1015</v>
+        <v>1011</v>
       </c>
       <c r="E10" t="s">
-        <v>1068</v>
+        <v>1064</v>
       </c>
       <c r="F10" t="s">
-        <v>1100</v>
+        <v>1096</v>
       </c>
       <c r="G10" t="s">
         <v>118</v>
@@ -4413,7 +4404,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>959</v>
+        <v>955</v>
       </c>
       <c r="B11">
         <v>166578</v>
@@ -4422,7 +4413,7 @@
         <v>19</v>
       </c>
       <c r="D11" t="s">
-        <v>1016</v>
+        <v>1012</v>
       </c>
       <c r="E11" t="s">
         <v>311</v>
@@ -4436,7 +4427,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>960</v>
+        <v>956</v>
       </c>
       <c r="B12">
         <v>166569</v>
@@ -4445,21 +4436,21 @@
         <v>20</v>
       </c>
       <c r="D12" t="s">
-        <v>1017</v>
+        <v>1013</v>
       </c>
       <c r="E12" t="s">
-        <v>1069</v>
+        <v>1065</v>
       </c>
       <c r="F12" t="s">
-        <v>1101</v>
+        <v>1097</v>
       </c>
       <c r="G12" t="s">
-        <v>1146</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>961</v>
+        <v>957</v>
       </c>
       <c r="B13">
         <v>166734</v>
@@ -4468,21 +4459,21 @@
         <v>10</v>
       </c>
       <c r="D13" t="s">
-        <v>1018</v>
+        <v>1014</v>
       </c>
       <c r="E13" t="s">
         <v>74</v>
       </c>
       <c r="F13" t="s">
-        <v>1102</v>
+        <v>1098</v>
       </c>
       <c r="G13" t="s">
-        <v>1147</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>962</v>
+        <v>958</v>
       </c>
       <c r="B14">
         <v>166806</v>
@@ -4491,7 +4482,7 @@
         <v>11</v>
       </c>
       <c r="D14" t="s">
-        <v>1019</v>
+        <v>1015</v>
       </c>
       <c r="E14" t="s">
         <v>311</v>
@@ -4505,7 +4496,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>963</v>
+        <v>959</v>
       </c>
       <c r="B15">
         <v>166637</v>
@@ -4514,13 +4505,13 @@
         <v>12</v>
       </c>
       <c r="D15" t="s">
-        <v>1020</v>
+        <v>1016</v>
       </c>
       <c r="E15" t="s">
-        <v>1070</v>
+        <v>1066</v>
       </c>
       <c r="F15" t="s">
-        <v>1103</v>
+        <v>1099</v>
       </c>
       <c r="G15" t="s">
         <v>118</v>
@@ -4528,7 +4519,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>964</v>
+        <v>960</v>
       </c>
       <c r="B16">
         <v>166648</v>
@@ -4537,13 +4528,13 @@
         <v>13</v>
       </c>
       <c r="D16" t="s">
-        <v>1021</v>
+        <v>1017</v>
       </c>
       <c r="E16" t="s">
         <v>340</v>
       </c>
       <c r="F16" t="s">
-        <v>908</v>
+        <v>904</v>
       </c>
       <c r="G16" t="s">
         <v>570</v>
@@ -4551,7 +4542,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>965</v>
+        <v>961</v>
       </c>
       <c r="B17">
         <v>166676</v>
@@ -4560,21 +4551,21 @@
         <v>14</v>
       </c>
       <c r="D17" t="s">
-        <v>1022</v>
+        <v>1018</v>
       </c>
       <c r="E17" t="s">
-        <v>1071</v>
+        <v>1067</v>
       </c>
       <c r="F17" t="s">
-        <v>1104</v>
+        <v>1100</v>
       </c>
       <c r="G17" t="s">
-        <v>1148</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>966</v>
+        <v>962</v>
       </c>
       <c r="B18">
         <v>166715</v>
@@ -4583,21 +4574,21 @@
         <v>15</v>
       </c>
       <c r="D18" t="s">
-        <v>1023</v>
+        <v>1019</v>
       </c>
       <c r="E18" t="s">
-        <v>1072</v>
+        <v>1068</v>
       </c>
       <c r="F18" t="s">
-        <v>1105</v>
+        <v>1101</v>
       </c>
       <c r="G18" t="s">
-        <v>1149</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>967</v>
+        <v>963</v>
       </c>
       <c r="B19">
         <v>166692</v>
@@ -4606,13 +4597,13 @@
         <v>16</v>
       </c>
       <c r="D19" t="s">
-        <v>1024</v>
+        <v>1020</v>
       </c>
       <c r="E19" t="s">
-        <v>1073</v>
+        <v>1069</v>
       </c>
       <c r="F19" t="s">
-        <v>1106</v>
+        <v>1102</v>
       </c>
       <c r="G19" t="s">
         <v>118</v>
@@ -4620,7 +4611,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>968</v>
+        <v>964</v>
       </c>
       <c r="B20">
         <v>166694</v>
@@ -4629,13 +4620,13 @@
         <v>17</v>
       </c>
       <c r="D20" t="s">
-        <v>1025</v>
+        <v>1021</v>
       </c>
       <c r="E20" t="s">
         <v>167</v>
       </c>
       <c r="F20" t="s">
-        <v>1107</v>
+        <v>1103</v>
       </c>
       <c r="G20" t="s">
         <v>118</v>
@@ -4643,7 +4634,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>969</v>
+        <v>965</v>
       </c>
       <c r="B21">
         <v>166709</v>
@@ -4652,21 +4643,21 @@
         <v>18</v>
       </c>
       <c r="D21" t="s">
-        <v>1026</v>
+        <v>1022</v>
       </c>
       <c r="E21" t="s">
-        <v>1074</v>
+        <v>1070</v>
       </c>
       <c r="F21" t="s">
-        <v>1108</v>
+        <v>1104</v>
       </c>
       <c r="G21" t="s">
-        <v>1150</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>970</v>
+        <v>966</v>
       </c>
       <c r="B22">
         <v>166717</v>
@@ -4675,21 +4666,21 @@
         <v>19</v>
       </c>
       <c r="D22" t="s">
-        <v>1027</v>
+        <v>1023</v>
       </c>
       <c r="E22" t="s">
-        <v>1075</v>
+        <v>1071</v>
       </c>
       <c r="F22" t="s">
-        <v>1109</v>
+        <v>1105</v>
       </c>
       <c r="G22" t="s">
-        <v>1151</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>971</v>
+        <v>967</v>
       </c>
       <c r="B23">
         <v>166751</v>
@@ -4698,21 +4689,21 @@
         <v>20</v>
       </c>
       <c r="D23" t="s">
-        <v>1028</v>
+        <v>1024</v>
       </c>
       <c r="E23" t="s">
         <v>326</v>
       </c>
       <c r="F23" t="s">
-        <v>1110</v>
+        <v>1106</v>
       </c>
       <c r="G23" t="s">
-        <v>1152</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>972</v>
+        <v>968</v>
       </c>
       <c r="B24">
         <v>166777</v>
@@ -4721,21 +4712,21 @@
         <v>10</v>
       </c>
       <c r="D24" t="s">
-        <v>1029</v>
+        <v>1025</v>
       </c>
       <c r="E24" t="s">
         <v>318</v>
       </c>
       <c r="F24" t="s">
-        <v>1111</v>
+        <v>1107</v>
       </c>
       <c r="G24" t="s">
-        <v>1153</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>973</v>
+        <v>969</v>
       </c>
       <c r="B25">
         <v>166789</v>
@@ -4744,7 +4735,7 @@
         <v>11</v>
       </c>
       <c r="D25" t="s">
-        <v>1030</v>
+        <v>1026</v>
       </c>
       <c r="E25" t="s">
         <v>311</v>
@@ -4758,7 +4749,7 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>974</v>
+        <v>970</v>
       </c>
       <c r="B26">
         <v>166791</v>
@@ -4767,21 +4758,21 @@
         <v>12</v>
       </c>
       <c r="D26" t="s">
-        <v>1031</v>
+        <v>1027</v>
       </c>
       <c r="E26" t="s">
-        <v>1076</v>
+        <v>1072</v>
       </c>
       <c r="F26" t="s">
-        <v>1112</v>
+        <v>1108</v>
       </c>
       <c r="G26" t="s">
-        <v>1154</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>975</v>
+        <v>971</v>
       </c>
       <c r="B27">
         <v>166819</v>
@@ -4790,21 +4781,21 @@
         <v>13</v>
       </c>
       <c r="D27" t="s">
-        <v>1032</v>
+        <v>1028</v>
       </c>
       <c r="E27" t="s">
         <v>84</v>
       </c>
       <c r="F27" t="s">
-        <v>924</v>
+        <v>920</v>
       </c>
       <c r="G27" t="s">
-        <v>948</v>
+        <v>944</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>976</v>
+        <v>972</v>
       </c>
       <c r="B28">
         <v>166527</v>
@@ -4813,21 +4804,21 @@
         <v>14</v>
       </c>
       <c r="D28" t="s">
-        <v>1033</v>
+        <v>1029</v>
       </c>
       <c r="E28" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="F28" t="s">
-        <v>1113</v>
+        <v>1109</v>
       </c>
       <c r="G28" t="s">
-        <v>1155</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>977</v>
+        <v>973</v>
       </c>
       <c r="B29">
         <v>166610</v>
@@ -4836,21 +4827,21 @@
         <v>15</v>
       </c>
       <c r="D29" t="s">
-        <v>1034</v>
+        <v>1030</v>
       </c>
       <c r="E29" t="s">
-        <v>1077</v>
+        <v>1073</v>
       </c>
       <c r="F29" t="s">
-        <v>1114</v>
+        <v>1110</v>
       </c>
       <c r="G29" t="s">
-        <v>1156</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>978</v>
+        <v>974</v>
       </c>
       <c r="B30">
         <v>166512</v>
@@ -4859,13 +4850,13 @@
         <v>16</v>
       </c>
       <c r="D30" t="s">
-        <v>1035</v>
+        <v>1031</v>
       </c>
       <c r="E30" t="s">
         <v>326</v>
       </c>
       <c r="F30" t="s">
-        <v>1115</v>
+        <v>1111</v>
       </c>
       <c r="G30" t="s">
         <v>118</v>
@@ -4873,7 +4864,7 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>979</v>
+        <v>975</v>
       </c>
       <c r="B31">
         <v>166526</v>
@@ -4882,13 +4873,13 @@
         <v>17</v>
       </c>
       <c r="D31" t="s">
-        <v>1036</v>
+        <v>1032</v>
       </c>
       <c r="E31" t="s">
-        <v>717</v>
+        <v>713</v>
       </c>
       <c r="F31" t="s">
-        <v>1116</v>
+        <v>1112</v>
       </c>
       <c r="G31" t="s">
         <v>118</v>
@@ -4896,7 +4887,7 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>980</v>
+        <v>976</v>
       </c>
       <c r="B32">
         <v>166530</v>
@@ -4905,13 +4896,13 @@
         <v>18</v>
       </c>
       <c r="D32" t="s">
-        <v>1037</v>
+        <v>1033</v>
       </c>
       <c r="E32" t="s">
-        <v>1078</v>
+        <v>1074</v>
       </c>
       <c r="F32" t="s">
-        <v>1117</v>
+        <v>1113</v>
       </c>
       <c r="G32" t="s">
         <v>118</v>
@@ -4919,7 +4910,7 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>981</v>
+        <v>977</v>
       </c>
       <c r="B33">
         <v>166602</v>
@@ -4928,13 +4919,13 @@
         <v>19</v>
       </c>
       <c r="D33" t="s">
-        <v>1038</v>
+        <v>1034</v>
       </c>
       <c r="E33" t="s">
-        <v>1079</v>
+        <v>1075</v>
       </c>
       <c r="F33" t="s">
-        <v>1118</v>
+        <v>1114</v>
       </c>
       <c r="G33" t="s">
         <v>118</v>
@@ -4942,7 +4933,7 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>982</v>
+        <v>978</v>
       </c>
       <c r="B34">
         <v>166605</v>
@@ -4951,13 +4942,13 @@
         <v>20</v>
       </c>
       <c r="D34" t="s">
-        <v>1039</v>
+        <v>1035</v>
       </c>
       <c r="E34" t="s">
-        <v>724</v>
+        <v>720</v>
       </c>
       <c r="F34" t="s">
-        <v>1119</v>
+        <v>1115</v>
       </c>
       <c r="G34" t="s">
         <v>118</v>
@@ -4965,7 +4956,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>983</v>
+        <v>979</v>
       </c>
       <c r="B35">
         <v>166614</v>
@@ -4974,21 +4965,21 @@
         <v>10</v>
       </c>
       <c r="D35" t="s">
-        <v>1040</v>
+        <v>1036</v>
       </c>
       <c r="E35" t="s">
-        <v>1185</v>
+        <v>1181</v>
       </c>
       <c r="F35" t="s">
-        <v>1186</v>
+        <v>1182</v>
       </c>
       <c r="G35" t="s">
-        <v>1157</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>984</v>
+        <v>980</v>
       </c>
       <c r="B36">
         <v>166618</v>
@@ -4997,13 +4988,13 @@
         <v>11</v>
       </c>
       <c r="D36" t="s">
-        <v>1041</v>
+        <v>1037</v>
       </c>
       <c r="E36" t="s">
-        <v>1078</v>
+        <v>1074</v>
       </c>
       <c r="F36" t="s">
-        <v>1120</v>
+        <v>1116</v>
       </c>
       <c r="G36" t="s">
         <v>118</v>
@@ -5011,7 +5002,7 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>985</v>
+        <v>981</v>
       </c>
       <c r="B37">
         <v>166620</v>
@@ -5020,21 +5011,21 @@
         <v>12</v>
       </c>
       <c r="D37" t="s">
-        <v>1042</v>
+        <v>1038</v>
       </c>
       <c r="E37" t="s">
         <v>172</v>
       </c>
       <c r="F37" t="s">
-        <v>1121</v>
+        <v>1117</v>
       </c>
       <c r="G37" t="s">
-        <v>1158</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>986</v>
+        <v>982</v>
       </c>
       <c r="B38">
         <v>166621</v>
@@ -5043,21 +5034,21 @@
         <v>13</v>
       </c>
       <c r="D38" t="s">
-        <v>1043</v>
+        <v>1039</v>
       </c>
       <c r="E38" t="s">
-        <v>1080</v>
+        <v>1076</v>
       </c>
       <c r="F38" t="s">
-        <v>1122</v>
+        <v>1118</v>
       </c>
       <c r="G38" t="s">
-        <v>1159</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>987</v>
+        <v>983</v>
       </c>
       <c r="B39">
         <v>166632</v>
@@ -5066,21 +5057,21 @@
         <v>14</v>
       </c>
       <c r="D39" t="s">
-        <v>1044</v>
+        <v>1040</v>
       </c>
       <c r="E39" t="s">
-        <v>1081</v>
+        <v>1077</v>
       </c>
       <c r="F39" t="s">
-        <v>1123</v>
+        <v>1119</v>
       </c>
       <c r="G39" t="s">
-        <v>1160</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>988</v>
+        <v>984</v>
       </c>
       <c r="B40">
         <v>166649</v>
@@ -5089,13 +5080,13 @@
         <v>15</v>
       </c>
       <c r="D40" t="s">
-        <v>1045</v>
+        <v>1041</v>
       </c>
       <c r="E40" t="s">
-        <v>1082</v>
+        <v>1078</v>
       </c>
       <c r="F40" t="s">
-        <v>1124</v>
+        <v>1120</v>
       </c>
       <c r="G40" t="s">
         <v>118</v>
@@ -5103,7 +5094,7 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>989</v>
+        <v>985</v>
       </c>
       <c r="B41">
         <v>166652</v>
@@ -5112,13 +5103,13 @@
         <v>16</v>
       </c>
       <c r="D41" t="s">
-        <v>1046</v>
+        <v>1042</v>
       </c>
       <c r="E41" t="s">
-        <v>1083</v>
+        <v>1079</v>
       </c>
       <c r="F41" t="s">
-        <v>1125</v>
+        <v>1121</v>
       </c>
       <c r="G41" t="s">
         <v>118</v>
@@ -5126,7 +5117,7 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>990</v>
+        <v>986</v>
       </c>
       <c r="B42">
         <v>166672</v>
@@ -5135,21 +5126,21 @@
         <v>17</v>
       </c>
       <c r="D42" t="s">
-        <v>1047</v>
+        <v>1043</v>
       </c>
       <c r="E42" t="s">
-        <v>1084</v>
+        <v>1080</v>
       </c>
       <c r="F42" t="s">
-        <v>1126</v>
+        <v>1122</v>
       </c>
       <c r="G42" t="s">
-        <v>1161</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>991</v>
+        <v>987</v>
       </c>
       <c r="B43">
         <v>166677</v>
@@ -5158,21 +5149,21 @@
         <v>18</v>
       </c>
       <c r="D43" t="s">
-        <v>1048</v>
+        <v>1044</v>
       </c>
       <c r="E43" t="s">
-        <v>717</v>
+        <v>713</v>
       </c>
       <c r="F43" t="s">
-        <v>1127</v>
+        <v>1123</v>
       </c>
       <c r="G43" t="s">
-        <v>1162</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>992</v>
+        <v>988</v>
       </c>
       <c r="B44">
         <v>166680</v>
@@ -5181,13 +5172,13 @@
         <v>19</v>
       </c>
       <c r="D44" t="s">
-        <v>1049</v>
+        <v>1045</v>
       </c>
       <c r="E44" t="s">
-        <v>1085</v>
+        <v>1081</v>
       </c>
       <c r="F44" t="s">
-        <v>1128</v>
+        <v>1124</v>
       </c>
       <c r="G44" t="s">
         <v>481</v>
@@ -5195,7 +5186,7 @@
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>993</v>
+        <v>989</v>
       </c>
       <c r="B45">
         <v>166718</v>
@@ -5204,21 +5195,21 @@
         <v>20</v>
       </c>
       <c r="D45" t="s">
-        <v>1050</v>
+        <v>1046</v>
       </c>
       <c r="E45" t="s">
-        <v>1086</v>
+        <v>1082</v>
       </c>
       <c r="F45" t="s">
-        <v>1129</v>
+        <v>1125</v>
       </c>
       <c r="G45" t="s">
-        <v>945</v>
+        <v>941</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>994</v>
+        <v>990</v>
       </c>
       <c r="B46">
         <v>166720</v>
@@ -5227,7 +5218,7 @@
         <v>10</v>
       </c>
       <c r="D46" t="s">
-        <v>1051</v>
+        <v>1047</v>
       </c>
       <c r="E46" t="s">
         <v>311</v>
@@ -5241,7 +5232,7 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>995</v>
+        <v>991</v>
       </c>
       <c r="B47">
         <v>166742</v>
@@ -5250,13 +5241,13 @@
         <v>11</v>
       </c>
       <c r="D47" t="s">
-        <v>1052</v>
+        <v>1048</v>
       </c>
       <c r="E47" t="s">
-        <v>713</v>
+        <v>709</v>
       </c>
       <c r="F47" t="s">
-        <v>1130</v>
+        <v>1126</v>
       </c>
       <c r="G47" t="s">
         <v>118</v>
@@ -5264,7 +5255,7 @@
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>996</v>
+        <v>992</v>
       </c>
       <c r="B48">
         <v>166752</v>
@@ -5273,13 +5264,13 @@
         <v>12</v>
       </c>
       <c r="D48" t="s">
-        <v>1053</v>
+        <v>1049</v>
       </c>
       <c r="E48" t="s">
-        <v>711</v>
+        <v>707</v>
       </c>
       <c r="F48" t="s">
-        <v>1131</v>
+        <v>1127</v>
       </c>
       <c r="G48" t="s">
         <v>118</v>
@@ -5287,7 +5278,7 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>997</v>
+        <v>993</v>
       </c>
       <c r="B49">
         <v>166761</v>
@@ -5296,21 +5287,21 @@
         <v>13</v>
       </c>
       <c r="D49" t="s">
-        <v>1054</v>
+        <v>1050</v>
       </c>
       <c r="E49" t="s">
-        <v>1087</v>
+        <v>1083</v>
       </c>
       <c r="F49" t="s">
-        <v>1132</v>
+        <v>1128</v>
       </c>
       <c r="G49" t="s">
-        <v>1163</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>998</v>
+        <v>994</v>
       </c>
       <c r="B50">
         <v>166772</v>
@@ -5319,21 +5310,21 @@
         <v>14</v>
       </c>
       <c r="D50" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="E50" t="s">
-        <v>1088</v>
+        <v>1084</v>
       </c>
       <c r="F50" t="s">
-        <v>1133</v>
+        <v>1129</v>
       </c>
       <c r="G50" t="s">
-        <v>1164</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>999</v>
+        <v>995</v>
       </c>
       <c r="B51">
         <v>166786</v>
@@ -5342,13 +5333,13 @@
         <v>15</v>
       </c>
       <c r="D51" t="s">
-        <v>1056</v>
+        <v>1052</v>
       </c>
       <c r="E51" t="s">
         <v>318</v>
       </c>
       <c r="F51" t="s">
-        <v>759</v>
+        <v>755</v>
       </c>
       <c r="G51" t="s">
         <v>118</v>
@@ -5356,7 +5347,7 @@
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>1000</v>
+        <v>996</v>
       </c>
       <c r="B52">
         <v>166815</v>
@@ -5365,21 +5356,21 @@
         <v>16</v>
       </c>
       <c r="D52" t="s">
-        <v>1057</v>
+        <v>1053</v>
       </c>
       <c r="E52" t="s">
         <v>306</v>
       </c>
       <c r="F52" t="s">
-        <v>1134</v>
+        <v>1130</v>
       </c>
       <c r="G52" t="s">
-        <v>1165</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>1001</v>
+        <v>997</v>
       </c>
       <c r="B53">
         <v>166816</v>
@@ -5388,13 +5379,13 @@
         <v>17</v>
       </c>
       <c r="D53" t="s">
-        <v>1058</v>
+        <v>1054</v>
       </c>
       <c r="E53" t="s">
-        <v>1089</v>
+        <v>1085</v>
       </c>
       <c r="F53" t="s">
-        <v>1135</v>
+        <v>1131</v>
       </c>
       <c r="G53" t="s">
         <v>118</v>
@@ -5402,7 +5393,7 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>1002</v>
+        <v>998</v>
       </c>
       <c r="B54">
         <v>166817</v>
@@ -5411,13 +5402,13 @@
         <v>18</v>
       </c>
       <c r="D54" t="s">
-        <v>1059</v>
+        <v>1055</v>
       </c>
       <c r="E54" t="s">
-        <v>886</v>
+        <v>882</v>
       </c>
       <c r="F54" t="s">
-        <v>1136</v>
+        <v>1132</v>
       </c>
       <c r="G54" t="s">
         <v>118</v>
@@ -5425,7 +5416,7 @@
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>1003</v>
+        <v>999</v>
       </c>
       <c r="B55">
         <v>167826</v>
@@ -5434,21 +5425,21 @@
         <v>19</v>
       </c>
       <c r="D55" t="s">
-        <v>1060</v>
+        <v>1056</v>
       </c>
       <c r="E55" t="s">
-        <v>1090</v>
+        <v>1086</v>
       </c>
       <c r="F55" t="s">
-        <v>1137</v>
+        <v>1133</v>
       </c>
       <c r="G55" t="s">
-        <v>1166</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>1004</v>
+        <v>1000</v>
       </c>
       <c r="B56">
         <v>167837</v>
@@ -5457,21 +5448,21 @@
         <v>20</v>
       </c>
       <c r="D56" t="s">
-        <v>1061</v>
+        <v>1057</v>
       </c>
       <c r="E56" t="s">
-        <v>1091</v>
+        <v>1087</v>
       </c>
       <c r="F56" t="s">
-        <v>1138</v>
+        <v>1134</v>
       </c>
       <c r="G56" t="s">
-        <v>1167</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>1005</v>
+        <v>1001</v>
       </c>
       <c r="B57">
         <v>170164</v>
@@ -5480,13 +5471,13 @@
         <v>10</v>
       </c>
       <c r="D57" t="s">
-        <v>1062</v>
+        <v>1058</v>
       </c>
       <c r="E57" t="s">
         <v>341</v>
       </c>
       <c r="F57" t="s">
-        <v>1139</v>
+        <v>1135</v>
       </c>
       <c r="G57" t="s">
         <v>118</v>
@@ -5494,7 +5485,7 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>1006</v>
+        <v>1002</v>
       </c>
       <c r="B58">
         <v>170518</v>
@@ -5503,16 +5494,16 @@
         <v>11</v>
       </c>
       <c r="D58" t="s">
-        <v>1063</v>
+        <v>1059</v>
       </c>
       <c r="E58" t="s">
-        <v>1191</v>
+        <v>1187</v>
       </c>
       <c r="F58" t="s">
-        <v>1190</v>
+        <v>1186</v>
       </c>
       <c r="G58" t="s">
-        <v>1168</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
@@ -5526,7 +5517,7 @@
         <v>12</v>
       </c>
       <c r="D59" t="s">
-        <v>1192</v>
+        <v>1188</v>
       </c>
       <c r="E59" t="s">
         <v>544</v>
@@ -6497,7 +6488,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="3" width="12.6640625" customWidth="1"/>
@@ -7187,10 +7178,10 @@
         <v>283</v>
       </c>
       <c r="E30" t="s">
-        <v>882</v>
+        <v>878</v>
       </c>
       <c r="F30" t="s">
-        <v>1179</v>
+        <v>1175</v>
       </c>
       <c r="G30" t="s">
         <v>400</v>
@@ -7607,6 +7598,29 @@
         <v>385</v>
       </c>
       <c r="G48" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A49" s="2">
+        <v>184</v>
+      </c>
+      <c r="B49">
+        <v>171868</v>
+      </c>
+      <c r="C49">
+        <v>6</v>
+      </c>
+      <c r="D49" t="s">
+        <v>1189</v>
+      </c>
+      <c r="E49" t="s">
+        <v>459</v>
+      </c>
+      <c r="F49" t="s">
+        <v>475</v>
+      </c>
+      <c r="G49" t="s">
         <v>118</v>
       </c>
     </row>
@@ -8106,7 +8120,7 @@
         <v>479</v>
       </c>
       <c r="G21" t="s">
-        <v>1184</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -8120,16 +8134,16 @@
         <v>17</v>
       </c>
       <c r="D22" t="s">
-        <v>1180</v>
+        <v>1176</v>
       </c>
       <c r="E22" t="s">
-        <v>1181</v>
+        <v>1177</v>
       </c>
       <c r="F22" t="s">
-        <v>1182</v>
+        <v>1178</v>
       </c>
       <c r="G22" t="s">
-        <v>1183</v>
+        <v>1179</v>
       </c>
     </row>
   </sheetData>
@@ -8605,7 +8619,7 @@
         <v>565</v>
       </c>
       <c r="G20" t="s">
-        <v>1187</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -8684,7 +8698,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="3" width="12.6640625" customWidth="1"/>
@@ -8727,13 +8741,13 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="E2" t="s">
         <v>172</v>
       </c>
       <c r="F2" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="G2" t="s">
         <v>118</v>
@@ -8750,16 +8764,16 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E3" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="F3" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="G3" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -8773,13 +8787,13 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="E4" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="F4" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="G4" t="s">
         <v>118</v>
@@ -8796,16 +8810,16 @@
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="E5" t="s">
         <v>172</v>
       </c>
       <c r="F5" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="G5" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -8819,16 +8833,16 @@
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="E6" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="F6" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="G6" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -8836,22 +8850,22 @@
         <v>587</v>
       </c>
       <c r="B7">
-        <v>166794</v>
+        <v>167882</v>
       </c>
       <c r="C7">
         <v>2</v>
       </c>
       <c r="D7" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="E7" t="s">
-        <v>605</v>
+        <v>167</v>
       </c>
       <c r="F7" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="G7" t="s">
-        <v>622</v>
+        <v>118</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -8859,22 +8873,22 @@
         <v>588</v>
       </c>
       <c r="B8">
-        <v>167882</v>
+        <v>166696</v>
       </c>
       <c r="C8">
         <v>3</v>
       </c>
       <c r="D8" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="E8" t="s">
-        <v>167</v>
+        <v>604</v>
       </c>
       <c r="F8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="G8" t="s">
-        <v>118</v>
+        <v>619</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -8882,22 +8896,22 @@
         <v>589</v>
       </c>
       <c r="B9">
-        <v>166696</v>
+        <v>166700</v>
       </c>
       <c r="C9">
         <v>4</v>
       </c>
       <c r="D9" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="E9" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="F9" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="G9" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -8905,44 +8919,21 @@
         <v>590</v>
       </c>
       <c r="B10">
-        <v>166700</v>
+        <v>166792</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="E10" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="F10" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="G10" t="s">
-        <v>624</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>591</v>
-      </c>
-      <c r="B11">
-        <v>166792</v>
-      </c>
-      <c r="C11">
-        <v>2</v>
-      </c>
-      <c r="D11" t="s">
-        <v>601</v>
-      </c>
-      <c r="E11" t="s">
-        <v>608</v>
-      </c>
-      <c r="F11" t="s">
-        <v>618</v>
-      </c>
-      <c r="G11" t="s">
         <v>118</v>
       </c>
     </row>
@@ -8987,7 +8978,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>625</v>
+        <v>621</v>
       </c>
       <c r="B2">
         <v>166462</v>
@@ -8996,13 +8987,13 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>666</v>
+        <v>662</v>
       </c>
       <c r="E2" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="F2" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="G2" t="s">
         <v>118</v>
@@ -9010,7 +9001,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>626</v>
+        <v>622</v>
       </c>
       <c r="B3">
         <v>166486</v>
@@ -9019,21 +9010,21 @@
         <v>6</v>
       </c>
       <c r="D3" t="s">
-        <v>667</v>
+        <v>663</v>
       </c>
       <c r="E3" t="s">
-        <v>707</v>
+        <v>703</v>
       </c>
       <c r="F3" t="s">
-        <v>729</v>
+        <v>725</v>
       </c>
       <c r="G3" t="s">
-        <v>764</v>
+        <v>760</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>627</v>
+        <v>623</v>
       </c>
       <c r="B4">
         <v>166545</v>
@@ -9042,13 +9033,13 @@
         <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>668</v>
+        <v>664</v>
       </c>
       <c r="E4" t="s">
-        <v>708</v>
+        <v>704</v>
       </c>
       <c r="F4" t="s">
-        <v>730</v>
+        <v>726</v>
       </c>
       <c r="G4" t="s">
         <v>118</v>
@@ -9056,7 +9047,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>628</v>
+        <v>624</v>
       </c>
       <c r="B5">
         <v>166557</v>
@@ -9065,21 +9056,21 @@
         <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>669</v>
+        <v>665</v>
       </c>
       <c r="E5" t="s">
-        <v>709</v>
+        <v>705</v>
       </c>
       <c r="F5" t="s">
-        <v>731</v>
+        <v>727</v>
       </c>
       <c r="G5" t="s">
-        <v>765</v>
+        <v>761</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>629</v>
+        <v>625</v>
       </c>
       <c r="B6">
         <v>166566</v>
@@ -9088,13 +9079,13 @@
         <v>9</v>
       </c>
       <c r="D6" t="s">
-        <v>670</v>
+        <v>666</v>
       </c>
       <c r="E6" t="s">
         <v>172</v>
       </c>
       <c r="F6" t="s">
-        <v>732</v>
+        <v>728</v>
       </c>
       <c r="G6" t="s">
         <v>118</v>
@@ -9102,7 +9093,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>630</v>
+        <v>626</v>
       </c>
       <c r="B7">
         <v>166600</v>
@@ -9111,13 +9102,13 @@
         <v>10</v>
       </c>
       <c r="D7" t="s">
-        <v>671</v>
+        <v>667</v>
       </c>
       <c r="E7" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="F7" t="s">
-        <v>733</v>
+        <v>729</v>
       </c>
       <c r="G7" t="s">
         <v>118</v>
@@ -9125,7 +9116,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>631</v>
+        <v>627</v>
       </c>
       <c r="B8">
         <v>166603</v>
@@ -9134,13 +9125,13 @@
         <v>11</v>
       </c>
       <c r="D8" t="s">
-        <v>672</v>
+        <v>668</v>
       </c>
       <c r="E8" t="s">
-        <v>710</v>
+        <v>706</v>
       </c>
       <c r="F8" t="s">
-        <v>734</v>
+        <v>730</v>
       </c>
       <c r="G8" t="s">
         <v>118</v>
@@ -9148,7 +9139,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>632</v>
+        <v>628</v>
       </c>
       <c r="B9">
         <v>166624</v>
@@ -9157,13 +9148,13 @@
         <v>12</v>
       </c>
       <c r="D9" t="s">
-        <v>673</v>
+        <v>669</v>
       </c>
       <c r="E9" t="s">
-        <v>711</v>
+        <v>707</v>
       </c>
       <c r="F9" t="s">
-        <v>735</v>
+        <v>731</v>
       </c>
       <c r="G9" t="s">
         <v>483</v>
@@ -9171,7 +9162,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>633</v>
+        <v>629</v>
       </c>
       <c r="B10">
         <v>166628</v>
@@ -9180,13 +9171,13 @@
         <v>13</v>
       </c>
       <c r="D10" t="s">
-        <v>674</v>
+        <v>670</v>
       </c>
       <c r="E10" t="s">
         <v>167</v>
       </c>
       <c r="F10" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="G10" t="s">
         <v>118</v>
@@ -9194,7 +9185,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>634</v>
+        <v>630</v>
       </c>
       <c r="B11">
         <v>166636</v>
@@ -9203,13 +9194,13 @@
         <v>14</v>
       </c>
       <c r="D11" t="s">
-        <v>675</v>
+        <v>671</v>
       </c>
       <c r="E11" t="s">
-        <v>712</v>
+        <v>708</v>
       </c>
       <c r="F11" t="s">
-        <v>736</v>
+        <v>732</v>
       </c>
       <c r="G11" t="s">
         <v>118</v>
@@ -9217,7 +9208,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>635</v>
+        <v>631</v>
       </c>
       <c r="B12">
         <v>166640</v>
@@ -9226,21 +9217,21 @@
         <v>15</v>
       </c>
       <c r="D12" t="s">
-        <v>676</v>
+        <v>672</v>
       </c>
       <c r="E12" t="s">
-        <v>713</v>
+        <v>709</v>
       </c>
       <c r="F12" t="s">
-        <v>737</v>
+        <v>733</v>
       </c>
       <c r="G12" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>636</v>
+        <v>632</v>
       </c>
       <c r="B13">
         <v>166668</v>
@@ -9249,13 +9240,13 @@
         <v>16</v>
       </c>
       <c r="D13" t="s">
-        <v>677</v>
+        <v>673</v>
       </c>
       <c r="E13" t="s">
         <v>458</v>
       </c>
       <c r="F13" t="s">
-        <v>738</v>
+        <v>734</v>
       </c>
       <c r="G13" t="s">
         <v>118</v>
@@ -9263,7 +9254,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>637</v>
+        <v>633</v>
       </c>
       <c r="B14">
         <v>166682</v>
@@ -9272,13 +9263,13 @@
         <v>17</v>
       </c>
       <c r="D14" t="s">
-        <v>678</v>
+        <v>674</v>
       </c>
       <c r="E14" t="s">
-        <v>1188</v>
+        <v>1184</v>
       </c>
       <c r="F14" t="s">
-        <v>1189</v>
+        <v>1185</v>
       </c>
       <c r="G14" t="s">
         <v>118</v>
@@ -9286,7 +9277,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>638</v>
+        <v>634</v>
       </c>
       <c r="B15">
         <v>166705</v>
@@ -9295,13 +9286,13 @@
         <v>18</v>
       </c>
       <c r="D15" t="s">
-        <v>679</v>
+        <v>675</v>
       </c>
       <c r="E15" t="s">
-        <v>714</v>
+        <v>710</v>
       </c>
       <c r="F15" t="s">
-        <v>740</v>
+        <v>736</v>
       </c>
       <c r="G15" t="s">
         <v>118</v>
@@ -9309,7 +9300,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>639</v>
+        <v>635</v>
       </c>
       <c r="B16">
         <v>166716</v>
@@ -9318,21 +9309,21 @@
         <v>19</v>
       </c>
       <c r="D16" t="s">
-        <v>680</v>
+        <v>676</v>
       </c>
       <c r="E16" t="s">
-        <v>715</v>
+        <v>711</v>
       </c>
       <c r="F16" t="s">
-        <v>741</v>
+        <v>737</v>
       </c>
       <c r="G16" t="s">
-        <v>765</v>
+        <v>761</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>640</v>
+        <v>636</v>
       </c>
       <c r="B17">
         <v>166743</v>
@@ -9341,13 +9332,13 @@
         <v>20</v>
       </c>
       <c r="D17" t="s">
-        <v>681</v>
+        <v>677</v>
       </c>
       <c r="E17" t="s">
         <v>167</v>
       </c>
       <c r="F17" t="s">
-        <v>742</v>
+        <v>738</v>
       </c>
       <c r="G17" t="s">
         <v>118</v>
@@ -9355,7 +9346,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>641</v>
+        <v>637</v>
       </c>
       <c r="B18">
         <v>166814</v>
@@ -9364,13 +9355,13 @@
         <v>5</v>
       </c>
       <c r="D18" t="s">
-        <v>682</v>
+        <v>678</v>
       </c>
       <c r="E18" t="s">
-        <v>716</v>
+        <v>712</v>
       </c>
       <c r="F18" t="s">
-        <v>743</v>
+        <v>739</v>
       </c>
       <c r="G18" t="s">
         <v>121</v>
@@ -9378,7 +9369,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>642</v>
+        <v>638</v>
       </c>
       <c r="B19">
         <v>166497</v>
@@ -9387,13 +9378,13 @@
         <v>6</v>
       </c>
       <c r="D19" t="s">
-        <v>683</v>
+        <v>679</v>
       </c>
       <c r="E19" t="s">
         <v>165</v>
       </c>
       <c r="F19" t="s">
-        <v>744</v>
+        <v>740</v>
       </c>
       <c r="G19" t="s">
         <v>118</v>
@@ -9401,7 +9392,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>643</v>
+        <v>639</v>
       </c>
       <c r="B20">
         <v>166733</v>
@@ -9410,13 +9401,13 @@
         <v>7</v>
       </c>
       <c r="D20" t="s">
-        <v>684</v>
+        <v>680</v>
       </c>
       <c r="E20" t="s">
-        <v>717</v>
+        <v>713</v>
       </c>
       <c r="F20" t="s">
-        <v>745</v>
+        <v>741</v>
       </c>
       <c r="G20" t="s">
         <v>118</v>
@@ -9424,7 +9415,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>644</v>
+        <v>640</v>
       </c>
       <c r="B21">
         <v>166496</v>
@@ -9433,13 +9424,13 @@
         <v>8</v>
       </c>
       <c r="D21" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="E21" t="s">
-        <v>718</v>
+        <v>714</v>
       </c>
       <c r="F21" t="s">
-        <v>746</v>
+        <v>742</v>
       </c>
       <c r="G21" t="s">
         <v>118</v>
@@ -9447,7 +9438,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>645</v>
+        <v>641</v>
       </c>
       <c r="B22">
         <v>166783</v>
@@ -9456,13 +9447,13 @@
         <v>9</v>
       </c>
       <c r="D22" t="s">
-        <v>686</v>
+        <v>682</v>
       </c>
       <c r="E22" t="s">
         <v>85</v>
       </c>
       <c r="F22" t="s">
-        <v>747</v>
+        <v>743</v>
       </c>
       <c r="G22" t="s">
         <v>118</v>
@@ -9470,7 +9461,7 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>646</v>
+        <v>642</v>
       </c>
       <c r="B23">
         <v>166468</v>
@@ -9479,13 +9470,13 @@
         <v>10</v>
       </c>
       <c r="D23" t="s">
-        <v>687</v>
+        <v>683</v>
       </c>
       <c r="E23" t="s">
         <v>162</v>
       </c>
       <c r="F23" t="s">
-        <v>748</v>
+        <v>744</v>
       </c>
       <c r="G23" t="s">
         <v>118</v>
@@ -9493,7 +9484,7 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>647</v>
+        <v>643</v>
       </c>
       <c r="B24">
         <v>166494</v>
@@ -9502,21 +9493,21 @@
         <v>11</v>
       </c>
       <c r="D24" t="s">
-        <v>688</v>
+        <v>684</v>
       </c>
       <c r="E24" t="s">
-        <v>712</v>
+        <v>708</v>
       </c>
       <c r="F24" t="s">
-        <v>749</v>
+        <v>745</v>
       </c>
       <c r="G24" t="s">
-        <v>767</v>
+        <v>763</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>648</v>
+        <v>644</v>
       </c>
       <c r="B25">
         <v>166509</v>
@@ -9525,21 +9516,21 @@
         <v>12</v>
       </c>
       <c r="D25" t="s">
-        <v>689</v>
+        <v>685</v>
       </c>
       <c r="E25" t="s">
-        <v>719</v>
+        <v>715</v>
       </c>
       <c r="F25" t="s">
-        <v>750</v>
+        <v>746</v>
       </c>
       <c r="G25" t="s">
-        <v>768</v>
+        <v>764</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>649</v>
+        <v>645</v>
       </c>
       <c r="B26">
         <v>166531</v>
@@ -9548,21 +9539,21 @@
         <v>13</v>
       </c>
       <c r="D26" t="s">
-        <v>690</v>
+        <v>686</v>
       </c>
       <c r="E26" t="s">
-        <v>720</v>
+        <v>716</v>
       </c>
       <c r="F26" t="s">
-        <v>751</v>
+        <v>747</v>
       </c>
       <c r="G26" t="s">
-        <v>769</v>
+        <v>765</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
       <c r="B27">
         <v>166532</v>
@@ -9571,13 +9562,13 @@
         <v>14</v>
       </c>
       <c r="D27" t="s">
-        <v>691</v>
+        <v>687</v>
       </c>
       <c r="E27" t="s">
         <v>543</v>
       </c>
       <c r="F27" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="G27" t="s">
         <v>118</v>
@@ -9585,7 +9576,7 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>651</v>
+        <v>647</v>
       </c>
       <c r="B28">
         <v>166559</v>
@@ -9594,21 +9585,21 @@
         <v>15</v>
       </c>
       <c r="D28" t="s">
-        <v>692</v>
+        <v>688</v>
       </c>
       <c r="E28" t="s">
         <v>545</v>
       </c>
       <c r="F28" t="s">
-        <v>753</v>
+        <v>749</v>
       </c>
       <c r="G28" t="s">
-        <v>770</v>
+        <v>766</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>652</v>
+        <v>648</v>
       </c>
       <c r="B29">
         <v>166564</v>
@@ -9617,13 +9608,13 @@
         <v>16</v>
       </c>
       <c r="D29" t="s">
-        <v>693</v>
+        <v>689</v>
       </c>
       <c r="E29" t="s">
         <v>167</v>
       </c>
       <c r="F29" t="s">
-        <v>742</v>
+        <v>738</v>
       </c>
       <c r="G29" t="s">
         <v>118</v>
@@ -9631,7 +9622,7 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>653</v>
+        <v>649</v>
       </c>
       <c r="B30">
         <v>166565</v>
@@ -9640,21 +9631,21 @@
         <v>17</v>
       </c>
       <c r="D30" t="s">
-        <v>694</v>
+        <v>690</v>
       </c>
       <c r="E30" t="s">
-        <v>721</v>
+        <v>717</v>
       </c>
       <c r="F30" t="s">
-        <v>754</v>
+        <v>750</v>
       </c>
       <c r="G30" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
       <c r="B31">
         <v>166606</v>
@@ -9663,13 +9654,13 @@
         <v>18</v>
       </c>
       <c r="D31" t="s">
-        <v>695</v>
+        <v>691</v>
       </c>
       <c r="E31" t="s">
-        <v>722</v>
+        <v>718</v>
       </c>
       <c r="F31" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="G31" t="s">
         <v>118</v>
@@ -9677,7 +9668,7 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>655</v>
+        <v>651</v>
       </c>
       <c r="B32">
         <v>166658</v>
@@ -9686,13 +9677,13 @@
         <v>19</v>
       </c>
       <c r="D32" t="s">
-        <v>696</v>
+        <v>692</v>
       </c>
       <c r="E32" t="s">
-        <v>723</v>
+        <v>719</v>
       </c>
       <c r="F32" t="s">
-        <v>756</v>
+        <v>752</v>
       </c>
       <c r="G32" t="s">
         <v>403</v>
@@ -9700,7 +9691,7 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
       <c r="B33">
         <v>166667</v>
@@ -9709,13 +9700,13 @@
         <v>20</v>
       </c>
       <c r="D33" t="s">
-        <v>697</v>
+        <v>693</v>
       </c>
       <c r="E33" t="s">
         <v>167</v>
       </c>
       <c r="F33" t="s">
-        <v>742</v>
+        <v>738</v>
       </c>
       <c r="G33" t="s">
         <v>118</v>
@@ -9723,7 +9714,7 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="B34">
         <v>166671</v>
@@ -9732,13 +9723,13 @@
         <v>5</v>
       </c>
       <c r="D34" t="s">
-        <v>698</v>
+        <v>694</v>
       </c>
       <c r="E34" t="s">
         <v>167</v>
       </c>
       <c r="F34" t="s">
-        <v>757</v>
+        <v>753</v>
       </c>
       <c r="G34" t="s">
         <v>118</v>
@@ -9746,7 +9737,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>658</v>
+        <v>654</v>
       </c>
       <c r="B35">
         <v>166684</v>
@@ -9755,21 +9746,21 @@
         <v>6</v>
       </c>
       <c r="D35" t="s">
-        <v>699</v>
+        <v>695</v>
       </c>
       <c r="E35" t="s">
-        <v>724</v>
+        <v>720</v>
       </c>
       <c r="F35" t="s">
-        <v>758</v>
+        <v>754</v>
       </c>
       <c r="G35" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
       <c r="B36">
         <v>166730</v>
@@ -9778,13 +9769,13 @@
         <v>7</v>
       </c>
       <c r="D36" t="s">
-        <v>700</v>
+        <v>696</v>
       </c>
       <c r="E36" t="s">
         <v>318</v>
       </c>
       <c r="F36" t="s">
-        <v>759</v>
+        <v>755</v>
       </c>
       <c r="G36" t="s">
         <v>118</v>
@@ -9792,7 +9783,7 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>660</v>
+        <v>656</v>
       </c>
       <c r="B37">
         <v>166736</v>
@@ -9801,13 +9792,13 @@
         <v>8</v>
       </c>
       <c r="D37" t="s">
-        <v>701</v>
+        <v>697</v>
       </c>
       <c r="E37" t="s">
-        <v>725</v>
+        <v>721</v>
       </c>
       <c r="F37" t="s">
-        <v>760</v>
+        <v>756</v>
       </c>
       <c r="G37" t="s">
         <v>118</v>
@@ -9815,7 +9806,7 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>661</v>
+        <v>657</v>
       </c>
       <c r="B38">
         <v>166739</v>
@@ -9824,21 +9815,21 @@
         <v>9</v>
       </c>
       <c r="D38" t="s">
-        <v>702</v>
+        <v>698</v>
       </c>
       <c r="E38" t="s">
-        <v>726</v>
+        <v>722</v>
       </c>
       <c r="F38" t="s">
-        <v>761</v>
+        <v>757</v>
       </c>
       <c r="G38" t="s">
-        <v>773</v>
+        <v>769</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>662</v>
+        <v>658</v>
       </c>
       <c r="B39">
         <v>166749</v>
@@ -9847,21 +9838,21 @@
         <v>10</v>
       </c>
       <c r="D39" t="s">
-        <v>703</v>
+        <v>699</v>
       </c>
       <c r="E39" t="s">
-        <v>727</v>
+        <v>723</v>
       </c>
       <c r="F39" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="G39" t="s">
-        <v>774</v>
+        <v>770</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="B40">
         <v>166766</v>
@@ -9870,13 +9861,13 @@
         <v>11</v>
       </c>
       <c r="D40" t="s">
-        <v>704</v>
+        <v>700</v>
       </c>
       <c r="E40" t="s">
         <v>88</v>
       </c>
       <c r="F40" t="s">
-        <v>739</v>
+        <v>735</v>
       </c>
       <c r="G40" t="s">
         <v>118</v>
@@ -9884,7 +9875,7 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>664</v>
+        <v>660</v>
       </c>
       <c r="B41">
         <v>167683</v>
@@ -9893,7 +9884,7 @@
         <v>12</v>
       </c>
       <c r="D41" t="s">
-        <v>705</v>
+        <v>701</v>
       </c>
       <c r="E41" t="s">
         <v>164</v>
@@ -9902,12 +9893,12 @@
         <v>182</v>
       </c>
       <c r="G41" t="s">
-        <v>775</v>
+        <v>771</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>665</v>
+        <v>661</v>
       </c>
       <c r="B42">
         <v>167825</v>
@@ -9916,16 +9907,16 @@
         <v>13</v>
       </c>
       <c r="D42" t="s">
-        <v>706</v>
+        <v>702</v>
       </c>
       <c r="E42" t="s">
-        <v>728</v>
+        <v>724</v>
       </c>
       <c r="F42" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="G42" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
@@ -9992,7 +9983,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="B2">
         <v>166521</v>
@@ -10001,13 +9992,13 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>820</v>
+        <v>816</v>
       </c>
       <c r="E2" t="s">
-        <v>863</v>
+        <v>859</v>
       </c>
       <c r="F2" t="s">
-        <v>890</v>
+        <v>886</v>
       </c>
       <c r="G2" t="s">
         <v>118</v>
@@ -10015,7 +10006,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="B3">
         <v>166516</v>
@@ -10024,21 +10015,21 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>821</v>
+        <v>817</v>
       </c>
       <c r="E3" t="s">
-        <v>863</v>
+        <v>859</v>
       </c>
       <c r="F3" t="s">
-        <v>891</v>
+        <v>887</v>
       </c>
       <c r="G3" t="s">
-        <v>928</v>
+        <v>924</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="B4">
         <v>166508</v>
@@ -10047,13 +10038,13 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>822</v>
+        <v>818</v>
       </c>
       <c r="E4" t="s">
-        <v>864</v>
+        <v>860</v>
       </c>
       <c r="F4" t="s">
-        <v>892</v>
+        <v>888</v>
       </c>
       <c r="G4" t="s">
         <v>118</v>
@@ -10061,7 +10052,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="B5">
         <v>166540</v>
@@ -10070,21 +10061,21 @@
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>823</v>
+        <v>819</v>
       </c>
       <c r="E5" t="s">
-        <v>865</v>
+        <v>861</v>
       </c>
       <c r="F5" t="s">
-        <v>893</v>
+        <v>889</v>
       </c>
       <c r="G5" t="s">
-        <v>929</v>
+        <v>925</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="B6">
         <v>166541</v>
@@ -10093,21 +10084,21 @@
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>824</v>
+        <v>820</v>
       </c>
       <c r="E6" t="s">
-        <v>866</v>
+        <v>862</v>
       </c>
       <c r="F6" t="s">
-        <v>894</v>
+        <v>890</v>
       </c>
       <c r="G6" t="s">
-        <v>930</v>
+        <v>926</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>782</v>
+        <v>778</v>
       </c>
       <c r="B7">
         <v>166561</v>
@@ -10116,21 +10107,21 @@
         <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>825</v>
+        <v>821</v>
       </c>
       <c r="E7" t="s">
-        <v>867</v>
+        <v>863</v>
       </c>
       <c r="F7" t="s">
         <v>368</v>
       </c>
       <c r="G7" t="s">
-        <v>931</v>
+        <v>927</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>783</v>
+        <v>779</v>
       </c>
       <c r="B8">
         <v>166619</v>
@@ -10139,21 +10130,21 @@
         <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>826</v>
+        <v>822</v>
       </c>
       <c r="E8" t="s">
-        <v>868</v>
+        <v>864</v>
       </c>
       <c r="F8" t="s">
-        <v>895</v>
+        <v>891</v>
       </c>
       <c r="G8" t="s">
-        <v>932</v>
+        <v>928</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>784</v>
+        <v>780</v>
       </c>
       <c r="B9">
         <v>166623</v>
@@ -10162,13 +10153,13 @@
         <v>8</v>
       </c>
       <c r="D9" t="s">
-        <v>827</v>
+        <v>823</v>
       </c>
       <c r="E9" t="s">
-        <v>869</v>
+        <v>865</v>
       </c>
       <c r="F9" t="s">
-        <v>896</v>
+        <v>892</v>
       </c>
       <c r="G9" t="s">
         <v>118</v>
@@ -10176,7 +10167,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>785</v>
+        <v>781</v>
       </c>
       <c r="B10">
         <v>166630</v>
@@ -10185,13 +10176,13 @@
         <v>9</v>
       </c>
       <c r="D10" t="s">
-        <v>828</v>
+        <v>824</v>
       </c>
       <c r="E10" t="s">
-        <v>870</v>
+        <v>866</v>
       </c>
       <c r="F10" t="s">
-        <v>897</v>
+        <v>893</v>
       </c>
       <c r="G10" t="s">
         <v>118</v>
@@ -10199,7 +10190,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>786</v>
+        <v>782</v>
       </c>
       <c r="B11">
         <v>166673</v>
@@ -10208,21 +10199,21 @@
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>829</v>
+        <v>825</v>
       </c>
       <c r="E11" t="s">
-        <v>871</v>
+        <v>867</v>
       </c>
       <c r="F11" t="s">
-        <v>898</v>
+        <v>894</v>
       </c>
       <c r="G11" t="s">
-        <v>933</v>
+        <v>929</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>787</v>
+        <v>783</v>
       </c>
       <c r="B12">
         <v>166675</v>
@@ -10231,21 +10222,21 @@
         <v>2</v>
       </c>
       <c r="D12" t="s">
-        <v>830</v>
+        <v>826</v>
       </c>
       <c r="E12" t="s">
-        <v>871</v>
+        <v>867</v>
       </c>
       <c r="F12" t="s">
-        <v>898</v>
+        <v>894</v>
       </c>
       <c r="G12" t="s">
-        <v>933</v>
+        <v>929</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>788</v>
+        <v>784</v>
       </c>
       <c r="B13">
         <v>166710</v>
@@ -10254,7 +10245,7 @@
         <v>3</v>
       </c>
       <c r="D13" t="s">
-        <v>831</v>
+        <v>827</v>
       </c>
       <c r="E13" t="s">
         <v>311</v>
@@ -10268,7 +10259,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>789</v>
+        <v>785</v>
       </c>
       <c r="B14">
         <v>166711</v>
@@ -10277,21 +10268,21 @@
         <v>4</v>
       </c>
       <c r="D14" t="s">
-        <v>832</v>
+        <v>828</v>
       </c>
       <c r="E14" t="s">
-        <v>872</v>
+        <v>868</v>
       </c>
       <c r="F14" t="s">
-        <v>899</v>
+        <v>895</v>
       </c>
       <c r="G14" t="s">
-        <v>934</v>
+        <v>930</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>790</v>
+        <v>786</v>
       </c>
       <c r="B15">
         <v>166755</v>
@@ -10300,13 +10291,13 @@
         <v>5</v>
       </c>
       <c r="D15" t="s">
-        <v>833</v>
+        <v>829</v>
       </c>
       <c r="E15" t="s">
         <v>172</v>
       </c>
       <c r="F15" t="s">
-        <v>900</v>
+        <v>896</v>
       </c>
       <c r="G15" t="s">
         <v>118</v>
@@ -10314,7 +10305,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>791</v>
+        <v>787</v>
       </c>
       <c r="B16">
         <v>166757</v>
@@ -10323,21 +10314,21 @@
         <v>6</v>
       </c>
       <c r="D16" t="s">
-        <v>834</v>
+        <v>830</v>
       </c>
       <c r="E16" t="s">
-        <v>873</v>
+        <v>869</v>
       </c>
       <c r="F16" t="s">
-        <v>901</v>
+        <v>897</v>
       </c>
       <c r="G16" t="s">
-        <v>935</v>
+        <v>931</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>792</v>
+        <v>788</v>
       </c>
       <c r="B17">
         <v>167481</v>
@@ -10346,13 +10337,13 @@
         <v>7</v>
       </c>
       <c r="D17" t="s">
-        <v>835</v>
+        <v>831</v>
       </c>
       <c r="E17" t="s">
-        <v>874</v>
+        <v>870</v>
       </c>
       <c r="F17" t="s">
-        <v>902</v>
+        <v>898</v>
       </c>
       <c r="G17" t="s">
         <v>114</v>
@@ -10360,7 +10351,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>793</v>
+        <v>789</v>
       </c>
       <c r="B18">
         <v>167793</v>
@@ -10369,13 +10360,13 @@
         <v>8</v>
       </c>
       <c r="D18" t="s">
-        <v>836</v>
+        <v>832</v>
       </c>
       <c r="E18" t="s">
         <v>162</v>
       </c>
       <c r="F18" t="s">
-        <v>903</v>
+        <v>899</v>
       </c>
       <c r="G18" t="s">
         <v>118</v>
@@ -10383,7 +10374,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>794</v>
+        <v>790</v>
       </c>
       <c r="B19">
         <v>168287</v>
@@ -10392,21 +10383,21 @@
         <v>9</v>
       </c>
       <c r="D19" t="s">
-        <v>837</v>
+        <v>833</v>
       </c>
       <c r="E19" t="s">
-        <v>875</v>
+        <v>871</v>
       </c>
       <c r="F19" t="s">
-        <v>904</v>
+        <v>900</v>
       </c>
       <c r="G19" t="s">
-        <v>936</v>
+        <v>932</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>795</v>
+        <v>791</v>
       </c>
       <c r="B20">
         <v>166567</v>
@@ -10415,21 +10406,21 @@
         <v>1</v>
       </c>
       <c r="D20" t="s">
-        <v>838</v>
+        <v>834</v>
       </c>
       <c r="E20" t="s">
-        <v>876</v>
+        <v>872</v>
       </c>
       <c r="F20" t="s">
-        <v>905</v>
+        <v>901</v>
       </c>
       <c r="G20" t="s">
-        <v>937</v>
+        <v>933</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>796</v>
+        <v>792</v>
       </c>
       <c r="B21">
         <v>166538</v>
@@ -10438,21 +10429,21 @@
         <v>2</v>
       </c>
       <c r="D21" t="s">
-        <v>839</v>
+        <v>835</v>
       </c>
       <c r="E21" t="s">
-        <v>877</v>
+        <v>873</v>
       </c>
       <c r="F21" t="s">
-        <v>906</v>
+        <v>902</v>
       </c>
       <c r="G21" t="s">
-        <v>938</v>
+        <v>934</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>797</v>
+        <v>793</v>
       </c>
       <c r="B22">
         <v>166678</v>
@@ -10461,21 +10452,21 @@
         <v>3</v>
       </c>
       <c r="D22" t="s">
-        <v>840</v>
+        <v>836</v>
       </c>
       <c r="E22" t="s">
-        <v>878</v>
+        <v>874</v>
       </c>
       <c r="F22" t="s">
-        <v>907</v>
+        <v>903</v>
       </c>
       <c r="G22" t="s">
-        <v>933</v>
+        <v>929</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>798</v>
+        <v>794</v>
       </c>
       <c r="B23">
         <v>167682</v>
@@ -10484,13 +10475,13 @@
         <v>4</v>
       </c>
       <c r="D23" t="s">
-        <v>841</v>
+        <v>837</v>
       </c>
       <c r="E23" t="s">
         <v>340</v>
       </c>
       <c r="F23" t="s">
-        <v>908</v>
+        <v>904</v>
       </c>
       <c r="G23" t="s">
         <v>570</v>
@@ -10498,7 +10489,7 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>799</v>
+        <v>795</v>
       </c>
       <c r="B24">
         <v>166529</v>
@@ -10507,21 +10498,21 @@
         <v>5</v>
       </c>
       <c r="D24" t="s">
-        <v>842</v>
+        <v>838</v>
       </c>
       <c r="E24" t="s">
-        <v>879</v>
+        <v>875</v>
       </c>
       <c r="F24" t="s">
-        <v>909</v>
+        <v>905</v>
       </c>
       <c r="G24" t="s">
-        <v>939</v>
+        <v>935</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>800</v>
+        <v>796</v>
       </c>
       <c r="B25">
         <v>166472</v>
@@ -10530,21 +10521,21 @@
         <v>6</v>
       </c>
       <c r="D25" t="s">
-        <v>843</v>
+        <v>839</v>
       </c>
       <c r="E25" t="s">
-        <v>713</v>
+        <v>709</v>
       </c>
       <c r="F25" t="s">
-        <v>910</v>
+        <v>906</v>
       </c>
       <c r="G25" t="s">
-        <v>940</v>
+        <v>936</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>801</v>
+        <v>797</v>
       </c>
       <c r="B26">
         <v>166571</v>
@@ -10553,21 +10544,21 @@
         <v>7</v>
       </c>
       <c r="D26" t="s">
-        <v>844</v>
+        <v>840</v>
       </c>
       <c r="E26" t="s">
-        <v>880</v>
+        <v>876</v>
       </c>
       <c r="F26" t="s">
-        <v>911</v>
+        <v>907</v>
       </c>
       <c r="G26" t="s">
-        <v>941</v>
+        <v>937</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>802</v>
+        <v>798</v>
       </c>
       <c r="B27">
         <v>166575</v>
@@ -10576,13 +10567,13 @@
         <v>8</v>
       </c>
       <c r="D27" t="s">
-        <v>845</v>
+        <v>841</v>
       </c>
       <c r="E27" t="s">
         <v>458</v>
       </c>
       <c r="F27" t="s">
-        <v>912</v>
+        <v>908</v>
       </c>
       <c r="G27" t="s">
         <v>118</v>
@@ -10590,7 +10581,7 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>803</v>
+        <v>799</v>
       </c>
       <c r="B28">
         <v>166590</v>
@@ -10599,21 +10590,21 @@
         <v>9</v>
       </c>
       <c r="D28" t="s">
-        <v>846</v>
+        <v>842</v>
       </c>
       <c r="E28" t="s">
-        <v>881</v>
+        <v>877</v>
       </c>
       <c r="F28" t="s">
-        <v>913</v>
+        <v>909</v>
       </c>
       <c r="G28" t="s">
-        <v>942</v>
+        <v>938</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>804</v>
+        <v>800</v>
       </c>
       <c r="B29">
         <v>166598</v>
@@ -10622,21 +10613,21 @@
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>847</v>
+        <v>843</v>
       </c>
       <c r="E29" t="s">
-        <v>864</v>
+        <v>860</v>
       </c>
       <c r="F29" t="s">
-        <v>914</v>
+        <v>910</v>
       </c>
       <c r="G29" t="s">
-        <v>936</v>
+        <v>932</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>805</v>
+        <v>801</v>
       </c>
       <c r="B30">
         <v>166629</v>
@@ -10645,13 +10636,13 @@
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>848</v>
+        <v>844</v>
       </c>
       <c r="E30" t="s">
-        <v>869</v>
+        <v>865</v>
       </c>
       <c r="F30" t="s">
-        <v>896</v>
+        <v>892</v>
       </c>
       <c r="G30" t="s">
         <v>118</v>
@@ -10659,7 +10650,7 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>806</v>
+        <v>802</v>
       </c>
       <c r="B31">
         <v>166650</v>
@@ -10668,21 +10659,21 @@
         <v>3</v>
       </c>
       <c r="D31" t="s">
-        <v>849</v>
+        <v>845</v>
       </c>
       <c r="E31" t="s">
-        <v>711</v>
+        <v>707</v>
       </c>
       <c r="F31" t="s">
-        <v>915</v>
+        <v>911</v>
       </c>
       <c r="G31" t="s">
-        <v>943</v>
+        <v>939</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>807</v>
+        <v>803</v>
       </c>
       <c r="B32">
         <v>166657</v>
@@ -10691,13 +10682,13 @@
         <v>4</v>
       </c>
       <c r="D32" t="s">
-        <v>850</v>
+        <v>846</v>
       </c>
       <c r="E32" t="s">
-        <v>882</v>
+        <v>878</v>
       </c>
       <c r="F32" t="s">
-        <v>916</v>
+        <v>912</v>
       </c>
       <c r="G32" t="s">
         <v>114</v>
@@ -10705,7 +10696,7 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>808</v>
+        <v>804</v>
       </c>
       <c r="B33">
         <v>166687</v>
@@ -10714,21 +10705,21 @@
         <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>851</v>
+        <v>847</v>
       </c>
       <c r="E33" t="s">
-        <v>883</v>
+        <v>879</v>
       </c>
       <c r="F33" t="s">
-        <v>917</v>
+        <v>913</v>
       </c>
       <c r="G33" t="s">
-        <v>944</v>
+        <v>940</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>809</v>
+        <v>805</v>
       </c>
       <c r="B34">
         <v>166691</v>
@@ -10737,7 +10728,7 @@
         <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>852</v>
+        <v>848</v>
       </c>
       <c r="E34" t="s">
         <v>336</v>
@@ -10751,7 +10742,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>810</v>
+        <v>806</v>
       </c>
       <c r="B35">
         <v>166708</v>
@@ -10760,13 +10751,13 @@
         <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>853</v>
+        <v>849</v>
       </c>
       <c r="E35" t="s">
-        <v>884</v>
+        <v>880</v>
       </c>
       <c r="F35" t="s">
-        <v>918</v>
+        <v>914</v>
       </c>
       <c r="G35" t="s">
         <v>118</v>
@@ -10774,7 +10765,7 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>811</v>
+        <v>807</v>
       </c>
       <c r="B36">
         <v>166719</v>
@@ -10783,21 +10774,21 @@
         <v>8</v>
       </c>
       <c r="D36" t="s">
-        <v>854</v>
+        <v>850</v>
       </c>
       <c r="E36" t="s">
-        <v>885</v>
+        <v>881</v>
       </c>
       <c r="F36" t="s">
-        <v>919</v>
+        <v>915</v>
       </c>
       <c r="G36" t="s">
-        <v>945</v>
+        <v>941</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>812</v>
+        <v>808</v>
       </c>
       <c r="B37">
         <v>166744</v>
@@ -10806,13 +10797,13 @@
         <v>9</v>
       </c>
       <c r="D37" t="s">
-        <v>855</v>
+        <v>851</v>
       </c>
       <c r="E37" t="s">
         <v>322</v>
       </c>
       <c r="F37" t="s">
-        <v>920</v>
+        <v>916</v>
       </c>
       <c r="G37" t="s">
         <v>118</v>
@@ -10820,7 +10811,7 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>813</v>
+        <v>809</v>
       </c>
       <c r="B38">
         <v>166746</v>
@@ -10829,21 +10820,21 @@
         <v>1</v>
       </c>
       <c r="D38" t="s">
-        <v>856</v>
+        <v>852</v>
       </c>
       <c r="E38" t="s">
-        <v>886</v>
+        <v>882</v>
       </c>
       <c r="F38" t="s">
-        <v>921</v>
+        <v>917</v>
       </c>
       <c r="G38" t="s">
-        <v>946</v>
+        <v>942</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="B39">
         <v>166753</v>
@@ -10852,21 +10843,21 @@
         <v>2</v>
       </c>
       <c r="D39" t="s">
-        <v>857</v>
+        <v>853</v>
       </c>
       <c r="E39" t="s">
         <v>312</v>
       </c>
       <c r="F39" t="s">
-        <v>922</v>
+        <v>918</v>
       </c>
       <c r="G39" t="s">
-        <v>947</v>
+        <v>943</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>815</v>
+        <v>811</v>
       </c>
       <c r="B40">
         <v>166779</v>
@@ -10875,13 +10866,13 @@
         <v>3</v>
       </c>
       <c r="D40" t="s">
-        <v>858</v>
+        <v>854</v>
       </c>
       <c r="E40" t="s">
-        <v>887</v>
+        <v>883</v>
       </c>
       <c r="F40" t="s">
-        <v>923</v>
+        <v>919</v>
       </c>
       <c r="G40" t="s">
         <v>118</v>
@@ -10889,7 +10880,7 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>816</v>
+        <v>812</v>
       </c>
       <c r="B41">
         <v>166818</v>
@@ -10898,21 +10889,21 @@
         <v>4</v>
       </c>
       <c r="D41" t="s">
-        <v>859</v>
+        <v>855</v>
       </c>
       <c r="E41" t="s">
         <v>84</v>
       </c>
       <c r="F41" t="s">
-        <v>924</v>
+        <v>920</v>
       </c>
       <c r="G41" t="s">
-        <v>948</v>
+        <v>944</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>817</v>
+        <v>813</v>
       </c>
       <c r="B42">
         <v>167482</v>
@@ -10921,13 +10912,13 @@
         <v>5</v>
       </c>
       <c r="D42" t="s">
-        <v>860</v>
+        <v>856</v>
       </c>
       <c r="E42" t="s">
-        <v>888</v>
+        <v>884</v>
       </c>
       <c r="F42" t="s">
-        <v>925</v>
+        <v>921</v>
       </c>
       <c r="G42" t="s">
         <v>118</v>
@@ -10935,7 +10926,7 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>818</v>
+        <v>814</v>
       </c>
       <c r="B43">
         <v>167812</v>
@@ -10944,13 +10935,13 @@
         <v>6</v>
       </c>
       <c r="D43" t="s">
-        <v>861</v>
+        <v>857</v>
       </c>
       <c r="E43" t="s">
         <v>326</v>
       </c>
       <c r="F43" t="s">
-        <v>926</v>
+        <v>922</v>
       </c>
       <c r="G43" t="s">
         <v>118</v>
@@ -10958,7 +10949,7 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>819</v>
+        <v>815</v>
       </c>
       <c r="B44">
         <v>171332</v>
@@ -10967,16 +10958,16 @@
         <v>7</v>
       </c>
       <c r="D44" t="s">
-        <v>862</v>
+        <v>858</v>
       </c>
       <c r="E44" t="s">
-        <v>889</v>
+        <v>885</v>
       </c>
       <c r="F44" t="s">
-        <v>927</v>
+        <v>923</v>
       </c>
       <c r="G44" t="s">
-        <v>949</v>
+        <v>945</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Program updated, title 273
</commit_message>
<xml_diff>
--- a/pm2022/pm2022.xlsx
+++ b/pm2022/pm2022.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/galli/Documents/OrgConferenze/21PisaMeeting/pisameet/pm2022/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1F9749A-8B12-3543-A1FB-EC5559C257D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06519633-1D65-684B-9144-B42DF361114C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19360" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19360" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Program" sheetId="1" r:id="rId1"/>
@@ -1375,9 +1375,6 @@
     <t>Detection of inter-fraction morphological changes in particle therapy exploiting charged secondary fragments</t>
   </si>
   <si>
-    <t>The SciFi beam monitor</t>
-  </si>
-  <si>
     <t>The use of Low-Temperature Cofired Ceramics technology in Gas Electron Multiplier detectors</t>
   </si>
   <si>
@@ -3599,6 +3596,9 @@
   </si>
   <si>
     <t>Operational results with the pixelated timing Counter (pTC) of the MEGII experiment during the first year of physics data taking</t>
+  </si>
+  <si>
+    <t>Beam monitoring detectors for High Intensity Muon Beams</t>
   </si>
 </sst>
 </file>
@@ -4037,10 +4037,10 @@
         <v>13</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -4051,10 +4051,10 @@
         <v>14</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -4065,10 +4065,10 @@
         <v>15</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -4079,10 +4079,10 @@
         <v>16</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -4093,10 +4093,10 @@
         <v>17</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1167</v>
+        <v>1166</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -4107,10 +4107,10 @@
         <v>18</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -4121,10 +4121,10 @@
         <v>19</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -4135,10 +4135,10 @@
         <v>20</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -4149,10 +4149,10 @@
         <v>21</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
     </row>
   </sheetData>
@@ -4197,7 +4197,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="B2">
         <v>166461</v>
@@ -4206,21 +4206,21 @@
         <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="E2" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="F2" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="G2" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="B3">
         <v>166479</v>
@@ -4229,21 +4229,21 @@
         <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="E3" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="F3" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="G3" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="B4">
         <v>166522</v>
@@ -4252,21 +4252,21 @@
         <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="E4" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="F4" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
       <c r="G4" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="B5">
         <v>166488</v>
@@ -4275,21 +4275,21 @@
         <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="E5" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="F5" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="G5" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="B6">
         <v>166495</v>
@@ -4298,13 +4298,13 @@
         <v>14</v>
       </c>
       <c r="D6" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="E6" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="F6" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
       <c r="G6" t="s">
         <v>118</v>
@@ -4312,7 +4312,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="B7">
         <v>166520</v>
@@ -4321,21 +4321,21 @@
         <v>15</v>
       </c>
       <c r="D7" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="E7" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="F7" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="G7" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="B8">
         <v>166528</v>
@@ -4344,13 +4344,13 @@
         <v>16</v>
       </c>
       <c r="D8" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="E8" t="s">
         <v>312</v>
       </c>
       <c r="F8" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
       <c r="G8" t="s">
         <v>118</v>
@@ -4358,7 +4358,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="B9">
         <v>166523</v>
@@ -4367,21 +4367,21 @@
         <v>17</v>
       </c>
       <c r="D9" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="E9" t="s">
         <v>341</v>
       </c>
       <c r="F9" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
       <c r="G9" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="B10">
         <v>166570</v>
@@ -4390,13 +4390,13 @@
         <v>18</v>
       </c>
       <c r="D10" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="E10" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="F10" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
       <c r="G10" t="s">
         <v>118</v>
@@ -4404,7 +4404,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="B11">
         <v>166578</v>
@@ -4413,7 +4413,7 @@
         <v>19</v>
       </c>
       <c r="D11" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="E11" t="s">
         <v>311</v>
@@ -4427,7 +4427,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="B12">
         <v>166569</v>
@@ -4436,21 +4436,21 @@
         <v>20</v>
       </c>
       <c r="D12" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="E12" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="F12" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="G12" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="B13">
         <v>166734</v>
@@ -4459,21 +4459,21 @@
         <v>10</v>
       </c>
       <c r="D13" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="E13" t="s">
         <v>74</v>
       </c>
       <c r="F13" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
       <c r="G13" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="B14">
         <v>166806</v>
@@ -4482,7 +4482,7 @@
         <v>11</v>
       </c>
       <c r="D14" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="E14" t="s">
         <v>311</v>
@@ -4496,7 +4496,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="B15">
         <v>166637</v>
@@ -4505,13 +4505,13 @@
         <v>12</v>
       </c>
       <c r="D15" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="E15" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="F15" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
       <c r="G15" t="s">
         <v>118</v>
@@ -4519,7 +4519,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="B16">
         <v>166648</v>
@@ -4528,21 +4528,21 @@
         <v>13</v>
       </c>
       <c r="D16" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
       <c r="E16" t="s">
         <v>340</v>
       </c>
       <c r="F16" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="G16" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="B17">
         <v>166676</v>
@@ -4551,21 +4551,21 @@
         <v>14</v>
       </c>
       <c r="D17" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="E17" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="F17" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="G17" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="B18">
         <v>166715</v>
@@ -4574,21 +4574,21 @@
         <v>15</v>
       </c>
       <c r="D18" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="E18" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="F18" t="s">
-        <v>1101</v>
+        <v>1100</v>
       </c>
       <c r="G18" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="B19">
         <v>166692</v>
@@ -4597,13 +4597,13 @@
         <v>16</v>
       </c>
       <c r="D19" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="E19" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="F19" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
       <c r="G19" t="s">
         <v>118</v>
@@ -4611,7 +4611,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="B20">
         <v>166694</v>
@@ -4620,13 +4620,13 @@
         <v>17</v>
       </c>
       <c r="D20" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="E20" t="s">
         <v>167</v>
       </c>
       <c r="F20" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="G20" t="s">
         <v>118</v>
@@ -4634,7 +4634,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="B21">
         <v>166709</v>
@@ -4643,21 +4643,21 @@
         <v>18</v>
       </c>
       <c r="D21" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
       <c r="E21" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="F21" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
       <c r="G21" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="B22">
         <v>166717</v>
@@ -4666,21 +4666,21 @@
         <v>19</v>
       </c>
       <c r="D22" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="E22" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="F22" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
       <c r="G22" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="B23">
         <v>166751</v>
@@ -4689,21 +4689,21 @@
         <v>20</v>
       </c>
       <c r="D23" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="E23" t="s">
         <v>326</v>
       </c>
       <c r="F23" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
       <c r="G23" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="B24">
         <v>166777</v>
@@ -4712,21 +4712,21 @@
         <v>10</v>
       </c>
       <c r="D24" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="E24" t="s">
         <v>318</v>
       </c>
       <c r="F24" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="G24" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="B25">
         <v>166789</v>
@@ -4735,7 +4735,7 @@
         <v>11</v>
       </c>
       <c r="D25" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="E25" t="s">
         <v>311</v>
@@ -4749,7 +4749,7 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="B26">
         <v>166791</v>
@@ -4758,21 +4758,21 @@
         <v>12</v>
       </c>
       <c r="D26" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="E26" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
       <c r="F26" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="G26" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="B27">
         <v>166819</v>
@@ -4781,21 +4781,21 @@
         <v>13</v>
       </c>
       <c r="D27" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="E27" t="s">
         <v>84</v>
       </c>
       <c r="F27" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="G27" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="B28">
         <v>166527</v>
@@ -4804,21 +4804,21 @@
         <v>14</v>
       </c>
       <c r="D28" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="E28" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="F28" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="G28" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="B29">
         <v>166610</v>
@@ -4827,21 +4827,21 @@
         <v>15</v>
       </c>
       <c r="D29" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="E29" t="s">
-        <v>1073</v>
+        <v>1072</v>
       </c>
       <c r="F29" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="G29" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="B30">
         <v>166512</v>
@@ -4850,13 +4850,13 @@
         <v>16</v>
       </c>
       <c r="D30" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="E30" t="s">
         <v>326</v>
       </c>
       <c r="F30" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="G30" t="s">
         <v>118</v>
@@ -4864,7 +4864,7 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="B31">
         <v>166526</v>
@@ -4873,13 +4873,13 @@
         <v>17</v>
       </c>
       <c r="D31" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="E31" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="F31" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="G31" t="s">
         <v>118</v>
@@ -4887,7 +4887,7 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="B32">
         <v>166530</v>
@@ -4896,13 +4896,13 @@
         <v>18</v>
       </c>
       <c r="D32" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="E32" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
       <c r="F32" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="G32" t="s">
         <v>118</v>
@@ -4910,7 +4910,7 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="B33">
         <v>166602</v>
@@ -4919,13 +4919,13 @@
         <v>19</v>
       </c>
       <c r="D33" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="E33" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="F33" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="G33" t="s">
         <v>118</v>
@@ -4933,7 +4933,7 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="B34">
         <v>166605</v>
@@ -4942,13 +4942,13 @@
         <v>20</v>
       </c>
       <c r="D34" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="E34" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="F34" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
       <c r="G34" t="s">
         <v>118</v>
@@ -4956,7 +4956,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="B35">
         <v>166614</v>
@@ -4965,21 +4965,21 @@
         <v>10</v>
       </c>
       <c r="D35" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="E35" t="s">
+        <v>1180</v>
+      </c>
+      <c r="F35" t="s">
         <v>1181</v>
       </c>
-      <c r="F35" t="s">
-        <v>1182</v>
-      </c>
       <c r="G35" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="B36">
         <v>166618</v>
@@ -4988,13 +4988,13 @@
         <v>11</v>
       </c>
       <c r="D36" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="E36" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
       <c r="F36" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="G36" t="s">
         <v>118</v>
@@ -5002,7 +5002,7 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="B37">
         <v>166620</v>
@@ -5011,21 +5011,21 @@
         <v>12</v>
       </c>
       <c r="D37" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="E37" t="s">
         <v>172</v>
       </c>
       <c r="F37" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
       <c r="G37" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="B38">
         <v>166621</v>
@@ -5034,21 +5034,21 @@
         <v>13</v>
       </c>
       <c r="D38" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
       <c r="E38" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
       <c r="F38" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="G38" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="B39">
         <v>166632</v>
@@ -5057,21 +5057,21 @@
         <v>14</v>
       </c>
       <c r="D39" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
       <c r="E39" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="F39" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="G39" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="B40">
         <v>166649</v>
@@ -5080,13 +5080,13 @@
         <v>15</v>
       </c>
       <c r="D40" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
       <c r="E40" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="F40" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="G40" t="s">
         <v>118</v>
@@ -5094,7 +5094,7 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="B41">
         <v>166652</v>
@@ -5103,13 +5103,13 @@
         <v>16</v>
       </c>
       <c r="D41" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="E41" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="F41" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="G41" t="s">
         <v>118</v>
@@ -5117,7 +5117,7 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="B42">
         <v>166672</v>
@@ -5126,21 +5126,21 @@
         <v>17</v>
       </c>
       <c r="D42" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="E42" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="F42" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="G42" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="B43">
         <v>166677</v>
@@ -5149,21 +5149,21 @@
         <v>18</v>
       </c>
       <c r="D43" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="E43" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="F43" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="G43" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="B44">
         <v>166680</v>
@@ -5172,21 +5172,21 @@
         <v>19</v>
       </c>
       <c r="D44" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="E44" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="F44" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="G44" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="B45">
         <v>166718</v>
@@ -5195,21 +5195,21 @@
         <v>20</v>
       </c>
       <c r="D45" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="E45" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
       <c r="F45" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="G45" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="B46">
         <v>166720</v>
@@ -5218,7 +5218,7 @@
         <v>10</v>
       </c>
       <c r="D46" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="E46" t="s">
         <v>311</v>
@@ -5232,7 +5232,7 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="B47">
         <v>166742</v>
@@ -5241,13 +5241,13 @@
         <v>11</v>
       </c>
       <c r="D47" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="E47" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="F47" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="G47" t="s">
         <v>118</v>
@@ -5255,7 +5255,7 @@
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="B48">
         <v>166752</v>
@@ -5264,13 +5264,13 @@
         <v>12</v>
       </c>
       <c r="D48" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="E48" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="F48" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="G48" t="s">
         <v>118</v>
@@ -5278,7 +5278,7 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="B49">
         <v>166761</v>
@@ -5287,21 +5287,21 @@
         <v>13</v>
       </c>
       <c r="D49" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="E49" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="F49" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="G49" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="B50">
         <v>166772</v>
@@ -5310,21 +5310,21 @@
         <v>14</v>
       </c>
       <c r="D50" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="E50" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
       <c r="F50" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="G50" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="B51">
         <v>166786</v>
@@ -5333,13 +5333,13 @@
         <v>15</v>
       </c>
       <c r="D51" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="E51" t="s">
         <v>318</v>
       </c>
       <c r="F51" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G51" t="s">
         <v>118</v>
@@ -5347,7 +5347,7 @@
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="B52">
         <v>166815</v>
@@ -5356,21 +5356,21 @@
         <v>16</v>
       </c>
       <c r="D52" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="E52" t="s">
         <v>306</v>
       </c>
       <c r="F52" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="G52" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="B53">
         <v>166816</v>
@@ -5379,13 +5379,13 @@
         <v>17</v>
       </c>
       <c r="D53" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="E53" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="F53" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
       <c r="G53" t="s">
         <v>118</v>
@@ -5393,7 +5393,7 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="B54">
         <v>166817</v>
@@ -5402,13 +5402,13 @@
         <v>18</v>
       </c>
       <c r="D54" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="E54" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="F54" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
       <c r="G54" t="s">
         <v>118</v>
@@ -5416,7 +5416,7 @@
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="B55">
         <v>167826</v>
@@ -5425,21 +5425,21 @@
         <v>19</v>
       </c>
       <c r="D55" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="E55" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="F55" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="G55" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="B56">
         <v>167837</v>
@@ -5448,21 +5448,21 @@
         <v>20</v>
       </c>
       <c r="D56" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="E56" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
       <c r="F56" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="G56" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="B57">
         <v>170164</v>
@@ -5471,13 +5471,13 @@
         <v>10</v>
       </c>
       <c r="D57" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="E57" t="s">
         <v>341</v>
       </c>
       <c r="F57" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="G57" t="s">
         <v>118</v>
@@ -5485,7 +5485,7 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="B58">
         <v>170518</v>
@@ -5494,16 +5494,16 @@
         <v>11</v>
       </c>
       <c r="D58" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="E58" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="F58" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="G58" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
@@ -5517,16 +5517,16 @@
         <v>12</v>
       </c>
       <c r="D59" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="E59" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="F59" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="G59" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
   </sheetData>
@@ -7178,10 +7178,10 @@
         <v>283</v>
       </c>
       <c r="E30" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="F30" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="G30" t="s">
         <v>400</v>
@@ -7612,13 +7612,13 @@
         <v>6</v>
       </c>
       <c r="D49" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="E49" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="F49" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="G49" t="s">
         <v>118</v>
@@ -7677,10 +7677,10 @@
         <v>430</v>
       </c>
       <c r="E2" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="F2" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="G2" t="s">
         <v>118</v>
@@ -7700,10 +7700,10 @@
         <v>431</v>
       </c>
       <c r="E3" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F3" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="G3" t="s">
         <v>118</v>
@@ -7723,13 +7723,13 @@
         <v>432</v>
       </c>
       <c r="E4" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="F4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="G4" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -7749,10 +7749,10 @@
         <v>303</v>
       </c>
       <c r="F5" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="G5" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -7769,13 +7769,13 @@
         <v>434</v>
       </c>
       <c r="E6" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="F6" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="G6" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -7792,13 +7792,13 @@
         <v>435</v>
       </c>
       <c r="E7" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="F7" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="G7" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -7838,10 +7838,10 @@
         <v>437</v>
       </c>
       <c r="E9" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="F9" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="G9" t="s">
         <v>118</v>
@@ -7861,13 +7861,13 @@
         <v>438</v>
       </c>
       <c r="E10" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="F10" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="G10" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -7887,10 +7887,10 @@
         <v>164</v>
       </c>
       <c r="F11" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="G11" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -7910,7 +7910,7 @@
         <v>167</v>
       </c>
       <c r="F12" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="G12" t="s">
         <v>118</v>
@@ -7930,10 +7930,10 @@
         <v>441</v>
       </c>
       <c r="E13" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="F13" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="G13" t="s">
         <v>114</v>
@@ -7953,10 +7953,10 @@
         <v>442</v>
       </c>
       <c r="E14" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F14" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="G14" t="s">
         <v>118</v>
@@ -7979,7 +7979,7 @@
         <v>162</v>
       </c>
       <c r="F15" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="G15" t="s">
         <v>118</v>
@@ -7999,10 +7999,10 @@
         <v>444</v>
       </c>
       <c r="E16" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="F16" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="G16" t="s">
         <v>118</v>
@@ -8022,10 +8022,10 @@
         <v>445</v>
       </c>
       <c r="E17" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="F17" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="G17" t="s">
         <v>118</v>
@@ -8071,7 +8071,7 @@
         <v>309</v>
       </c>
       <c r="F19" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="G19" t="s">
         <v>118</v>
@@ -8088,16 +8088,16 @@
         <v>15</v>
       </c>
       <c r="D20" t="s">
-        <v>448</v>
+        <v>1189</v>
       </c>
       <c r="E20" t="s">
         <v>312</v>
       </c>
       <c r="F20" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="G20" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -8111,16 +8111,16 @@
         <v>16</v>
       </c>
       <c r="D21" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="E21" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="F21" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="G21" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -8134,16 +8134,16 @@
         <v>17</v>
       </c>
       <c r="D22" t="s">
+        <v>1175</v>
+      </c>
+      <c r="E22" t="s">
         <v>1176</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>1177</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>1178</v>
-      </c>
-      <c r="G22" t="s">
-        <v>1179</v>
       </c>
     </row>
   </sheetData>
@@ -8187,7 +8187,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B2">
         <v>166466</v>
@@ -8196,21 +8196,21 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="E2" t="s">
         <v>162</v>
       </c>
       <c r="F2" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="G2" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B3">
         <v>166467</v>
@@ -8219,21 +8219,21 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="E3" t="s">
         <v>74</v>
       </c>
       <c r="F3" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="G3" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B4">
         <v>166519</v>
@@ -8242,13 +8242,13 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="E4" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="F4" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="G4" t="s">
         <v>118</v>
@@ -8256,7 +8256,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B5">
         <v>166550</v>
@@ -8265,21 +8265,21 @@
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="E5" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="F5" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="G5" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="B6">
         <v>166645</v>
@@ -8288,21 +8288,21 @@
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="E6" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="F6" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="G6" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B7">
         <v>166643</v>
@@ -8311,21 +8311,21 @@
         <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="E7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F7" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="G7" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B8">
         <v>166685</v>
@@ -8334,21 +8334,21 @@
         <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="E8" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="F8" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="G8" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B9">
         <v>166810</v>
@@ -8357,21 +8357,21 @@
         <v>8</v>
       </c>
       <c r="D9" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="E9" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="F9" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="G9" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B10">
         <v>166740</v>
@@ -8380,7 +8380,7 @@
         <v>9</v>
       </c>
       <c r="D10" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="E10" t="s">
         <v>175</v>
@@ -8389,12 +8389,12 @@
         <v>192</v>
       </c>
       <c r="G10" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B11">
         <v>166754</v>
@@ -8403,13 +8403,13 @@
         <v>10</v>
       </c>
       <c r="D11" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="E11" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="F11" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G11" t="s">
         <v>118</v>
@@ -8417,7 +8417,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B12">
         <v>166775</v>
@@ -8426,13 +8426,13 @@
         <v>11</v>
       </c>
       <c r="D12" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="E12" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="F12" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="G12" t="s">
         <v>118</v>
@@ -8440,7 +8440,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B13">
         <v>166475</v>
@@ -8449,21 +8449,21 @@
         <v>12</v>
       </c>
       <c r="D13" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="E13" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="F13" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="G13" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B14">
         <v>166511</v>
@@ -8472,21 +8472,21 @@
         <v>13</v>
       </c>
       <c r="D14" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="E14" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="F14" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="G14" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="B15">
         <v>166518</v>
@@ -8495,13 +8495,13 @@
         <v>14</v>
       </c>
       <c r="D15" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="E15" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="F15" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="G15" t="s">
         <v>118</v>
@@ -8509,7 +8509,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B16">
         <v>166524</v>
@@ -8518,21 +8518,21 @@
         <v>15</v>
       </c>
       <c r="D16" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E16" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="F16" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="G16" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B17">
         <v>166525</v>
@@ -8541,13 +8541,13 @@
         <v>16</v>
       </c>
       <c r="D17" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="E17" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="F17" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="G17" t="s">
         <v>118</v>
@@ -8555,7 +8555,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B18">
         <v>166563</v>
@@ -8564,13 +8564,13 @@
         <v>17</v>
       </c>
       <c r="D18" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="E18" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="F18" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="G18" t="s">
         <v>114</v>
@@ -8578,7 +8578,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B19">
         <v>166608</v>
@@ -8587,21 +8587,21 @@
         <v>18</v>
       </c>
       <c r="D19" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="E19" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="F19" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="G19" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B20">
         <v>166659</v>
@@ -8610,21 +8610,21 @@
         <v>19</v>
       </c>
       <c r="D20" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="E20" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="F20" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="G20" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B21">
         <v>166664</v>
@@ -8633,13 +8633,13 @@
         <v>20</v>
       </c>
       <c r="D21" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="E21" t="s">
         <v>312</v>
       </c>
       <c r="F21" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="G21" t="s">
         <v>118</v>
@@ -8647,7 +8647,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="B22">
         <v>166727</v>
@@ -8656,21 +8656,21 @@
         <v>1</v>
       </c>
       <c r="D22" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="E22" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="F22" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="G22" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B23">
         <v>166738</v>
@@ -8679,13 +8679,13 @@
         <v>2</v>
       </c>
       <c r="D23" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="E23" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="F23" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="G23" t="s">
         <v>118</v>
@@ -8732,7 +8732,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="B2">
         <v>166656</v>
@@ -8741,13 +8741,13 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="E2" t="s">
         <v>172</v>
       </c>
       <c r="F2" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="G2" t="s">
         <v>118</v>
@@ -8755,7 +8755,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="B3">
         <v>166795</v>
@@ -8764,21 +8764,21 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="E3" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="F3" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="G3" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B4">
         <v>166674</v>
@@ -8787,13 +8787,13 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E4" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="F4" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="G4" t="s">
         <v>118</v>
@@ -8801,7 +8801,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="B5">
         <v>166582</v>
@@ -8810,21 +8810,21 @@
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="E5" t="s">
         <v>172</v>
       </c>
       <c r="F5" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="G5" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B6">
         <v>166679</v>
@@ -8833,21 +8833,21 @@
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="E6" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="F6" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="G6" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="B7">
         <v>167882</v>
@@ -8856,13 +8856,13 @@
         <v>2</v>
       </c>
       <c r="D7" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="E7" t="s">
         <v>167</v>
       </c>
       <c r="F7" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="G7" t="s">
         <v>118</v>
@@ -8870,7 +8870,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B8">
         <v>166696</v>
@@ -8879,21 +8879,21 @@
         <v>3</v>
       </c>
       <c r="D8" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="E8" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="F8" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="G8" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B9">
         <v>166700</v>
@@ -8902,21 +8902,21 @@
         <v>4</v>
       </c>
       <c r="D9" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="E9" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="F9" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="G9" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B10">
         <v>166792</v>
@@ -8925,13 +8925,13 @@
         <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="E10" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="F10" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="G10" t="s">
         <v>118</v>
@@ -8978,7 +8978,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="B2">
         <v>166462</v>
@@ -8987,13 +8987,13 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="E2" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="F2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="G2" t="s">
         <v>118</v>
@@ -9001,7 +9001,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B3">
         <v>166486</v>
@@ -9010,21 +9010,21 @@
         <v>6</v>
       </c>
       <c r="D3" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="E3" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="F3" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="G3" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B4">
         <v>166545</v>
@@ -9033,13 +9033,13 @@
         <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="E4" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="F4" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="G4" t="s">
         <v>118</v>
@@ -9047,7 +9047,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="B5">
         <v>166557</v>
@@ -9056,21 +9056,21 @@
         <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="E5" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="F5" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="G5" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B6">
         <v>166566</v>
@@ -9079,13 +9079,13 @@
         <v>9</v>
       </c>
       <c r="D6" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="E6" t="s">
         <v>172</v>
       </c>
       <c r="F6" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="G6" t="s">
         <v>118</v>
@@ -9093,7 +9093,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B7">
         <v>166600</v>
@@ -9102,13 +9102,13 @@
         <v>10</v>
       </c>
       <c r="D7" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="E7" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="F7" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="G7" t="s">
         <v>118</v>
@@ -9116,7 +9116,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="B8">
         <v>166603</v>
@@ -9125,13 +9125,13 @@
         <v>11</v>
       </c>
       <c r="D8" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="E8" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="F8" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="G8" t="s">
         <v>118</v>
@@ -9139,7 +9139,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="B9">
         <v>166624</v>
@@ -9148,21 +9148,21 @@
         <v>12</v>
       </c>
       <c r="D9" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="E9" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="F9" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="G9" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B10">
         <v>166628</v>
@@ -9171,13 +9171,13 @@
         <v>13</v>
       </c>
       <c r="D10" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="E10" t="s">
         <v>167</v>
       </c>
       <c r="F10" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="G10" t="s">
         <v>118</v>
@@ -9185,7 +9185,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="B11">
         <v>166636</v>
@@ -9194,13 +9194,13 @@
         <v>14</v>
       </c>
       <c r="D11" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="E11" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="F11" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="G11" t="s">
         <v>118</v>
@@ -9208,7 +9208,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B12">
         <v>166640</v>
@@ -9217,21 +9217,21 @@
         <v>15</v>
       </c>
       <c r="D12" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="E12" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="F12" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="G12" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B13">
         <v>166668</v>
@@ -9240,13 +9240,13 @@
         <v>16</v>
       </c>
       <c r="D13" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="E13" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F13" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="G13" t="s">
         <v>118</v>
@@ -9254,7 +9254,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="B14">
         <v>166682</v>
@@ -9263,13 +9263,13 @@
         <v>17</v>
       </c>
       <c r="D14" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="E14" t="s">
+        <v>1183</v>
+      </c>
+      <c r="F14" t="s">
         <v>1184</v>
-      </c>
-      <c r="F14" t="s">
-        <v>1185</v>
       </c>
       <c r="G14" t="s">
         <v>118</v>
@@ -9277,7 +9277,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B15">
         <v>166705</v>
@@ -9286,13 +9286,13 @@
         <v>18</v>
       </c>
       <c r="D15" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="E15" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="F15" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="G15" t="s">
         <v>118</v>
@@ -9300,7 +9300,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B16">
         <v>166716</v>
@@ -9309,21 +9309,21 @@
         <v>19</v>
       </c>
       <c r="D16" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="E16" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="F16" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="G16" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="B17">
         <v>166743</v>
@@ -9332,13 +9332,13 @@
         <v>20</v>
       </c>
       <c r="D17" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="E17" t="s">
         <v>167</v>
       </c>
       <c r="F17" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="G17" t="s">
         <v>118</v>
@@ -9346,7 +9346,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B18">
         <v>166814</v>
@@ -9355,13 +9355,13 @@
         <v>5</v>
       </c>
       <c r="D18" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="E18" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="F18" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="G18" t="s">
         <v>121</v>
@@ -9369,7 +9369,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="B19">
         <v>166497</v>
@@ -9378,13 +9378,13 @@
         <v>6</v>
       </c>
       <c r="D19" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="E19" t="s">
         <v>165</v>
       </c>
       <c r="F19" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="G19" t="s">
         <v>118</v>
@@ -9392,7 +9392,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="B20">
         <v>166733</v>
@@ -9401,13 +9401,13 @@
         <v>7</v>
       </c>
       <c r="D20" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="E20" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="F20" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="G20" t="s">
         <v>118</v>
@@ -9415,7 +9415,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="B21">
         <v>166496</v>
@@ -9424,13 +9424,13 @@
         <v>8</v>
       </c>
       <c r="D21" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="E21" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="F21" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="G21" t="s">
         <v>118</v>
@@ -9438,7 +9438,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="B22">
         <v>166783</v>
@@ -9447,13 +9447,13 @@
         <v>9</v>
       </c>
       <c r="D22" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E22" t="s">
         <v>85</v>
       </c>
       <c r="F22" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="G22" t="s">
         <v>118</v>
@@ -9461,7 +9461,7 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B23">
         <v>166468</v>
@@ -9470,13 +9470,13 @@
         <v>10</v>
       </c>
       <c r="D23" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E23" t="s">
         <v>162</v>
       </c>
       <c r="F23" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="G23" t="s">
         <v>118</v>
@@ -9484,7 +9484,7 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B24">
         <v>166494</v>
@@ -9493,21 +9493,21 @@
         <v>11</v>
       </c>
       <c r="D24" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="E24" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="F24" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="G24" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B25">
         <v>166509</v>
@@ -9516,21 +9516,21 @@
         <v>12</v>
       </c>
       <c r="D25" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="E25" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="F25" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="G25" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B26">
         <v>166531</v>
@@ -9539,21 +9539,21 @@
         <v>13</v>
       </c>
       <c r="D26" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="E26" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="F26" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="G26" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B27">
         <v>166532</v>
@@ -9562,13 +9562,13 @@
         <v>14</v>
       </c>
       <c r="D27" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E27" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="F27" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="G27" t="s">
         <v>118</v>
@@ -9576,7 +9576,7 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B28">
         <v>166559</v>
@@ -9585,21 +9585,21 @@
         <v>15</v>
       </c>
       <c r="D28" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="E28" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="F28" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="G28" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="B29">
         <v>166564</v>
@@ -9608,13 +9608,13 @@
         <v>16</v>
       </c>
       <c r="D29" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="E29" t="s">
         <v>167</v>
       </c>
       <c r="F29" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="G29" t="s">
         <v>118</v>
@@ -9622,7 +9622,7 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B30">
         <v>166565</v>
@@ -9631,21 +9631,21 @@
         <v>17</v>
       </c>
       <c r="D30" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="E30" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="F30" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="G30" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B31">
         <v>166606</v>
@@ -9654,13 +9654,13 @@
         <v>18</v>
       </c>
       <c r="D31" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="E31" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="F31" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="G31" t="s">
         <v>118</v>
@@ -9668,7 +9668,7 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="B32">
         <v>166658</v>
@@ -9677,13 +9677,13 @@
         <v>19</v>
       </c>
       <c r="D32" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="E32" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="F32" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="G32" t="s">
         <v>403</v>
@@ -9691,7 +9691,7 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="B33">
         <v>166667</v>
@@ -9700,13 +9700,13 @@
         <v>20</v>
       </c>
       <c r="D33" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="E33" t="s">
         <v>167</v>
       </c>
       <c r="F33" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="G33" t="s">
         <v>118</v>
@@ -9714,7 +9714,7 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B34">
         <v>166671</v>
@@ -9723,13 +9723,13 @@
         <v>5</v>
       </c>
       <c r="D34" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="E34" t="s">
         <v>167</v>
       </c>
       <c r="F34" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="G34" t="s">
         <v>118</v>
@@ -9737,7 +9737,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="B35">
         <v>166684</v>
@@ -9746,21 +9746,21 @@
         <v>6</v>
       </c>
       <c r="D35" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E35" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="F35" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="G35" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B36">
         <v>166730</v>
@@ -9769,13 +9769,13 @@
         <v>7</v>
       </c>
       <c r="D36" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="E36" t="s">
         <v>318</v>
       </c>
       <c r="F36" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G36" t="s">
         <v>118</v>
@@ -9783,7 +9783,7 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="B37">
         <v>166736</v>
@@ -9792,13 +9792,13 @@
         <v>8</v>
       </c>
       <c r="D37" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="E37" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="F37" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="G37" t="s">
         <v>118</v>
@@ -9806,7 +9806,7 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B38">
         <v>166739</v>
@@ -9815,21 +9815,21 @@
         <v>9</v>
       </c>
       <c r="D38" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="E38" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="F38" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="G38" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="B39">
         <v>166749</v>
@@ -9838,21 +9838,21 @@
         <v>10</v>
       </c>
       <c r="D39" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="E39" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="F39" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="G39" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B40">
         <v>166766</v>
@@ -9861,13 +9861,13 @@
         <v>11</v>
       </c>
       <c r="D40" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="E40" t="s">
         <v>88</v>
       </c>
       <c r="F40" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="G40" t="s">
         <v>118</v>
@@ -9875,7 +9875,7 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B41">
         <v>167683</v>
@@ -9884,7 +9884,7 @@
         <v>12</v>
       </c>
       <c r="D41" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="E41" t="s">
         <v>164</v>
@@ -9893,12 +9893,12 @@
         <v>182</v>
       </c>
       <c r="G41" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="B42">
         <v>167825</v>
@@ -9907,16 +9907,16 @@
         <v>13</v>
       </c>
       <c r="D42" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="E42" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="F42" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="G42" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
@@ -9983,7 +9983,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="B2">
         <v>166521</v>
@@ -9992,13 +9992,13 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="E2" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="F2" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="G2" t="s">
         <v>118</v>
@@ -10006,7 +10006,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="B3">
         <v>166516</v>
@@ -10015,21 +10015,21 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="E3" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="F3" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="G3" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="B4">
         <v>166508</v>
@@ -10038,13 +10038,13 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="E4" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="F4" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="G4" t="s">
         <v>118</v>
@@ -10052,7 +10052,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="B5">
         <v>166540</v>
@@ -10061,21 +10061,21 @@
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="E5" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="F5" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="G5" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="B6">
         <v>166541</v>
@@ -10084,21 +10084,21 @@
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="E6" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="F6" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="G6" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="B7">
         <v>166561</v>
@@ -10107,21 +10107,21 @@
         <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="E7" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="F7" t="s">
         <v>368</v>
       </c>
       <c r="G7" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="B8">
         <v>166619</v>
@@ -10130,21 +10130,21 @@
         <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="E8" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="F8" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="G8" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="B9">
         <v>166623</v>
@@ -10153,13 +10153,13 @@
         <v>8</v>
       </c>
       <c r="D9" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="E9" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="F9" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="G9" t="s">
         <v>118</v>
@@ -10167,7 +10167,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="B10">
         <v>166630</v>
@@ -10176,13 +10176,13 @@
         <v>9</v>
       </c>
       <c r="D10" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="E10" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="F10" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G10" t="s">
         <v>118</v>
@@ -10190,7 +10190,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="B11">
         <v>166673</v>
@@ -10199,21 +10199,21 @@
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="E11" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="F11" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="G11" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="B12">
         <v>166675</v>
@@ -10222,21 +10222,21 @@
         <v>2</v>
       </c>
       <c r="D12" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="E12" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="F12" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="G12" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="B13">
         <v>166710</v>
@@ -10245,7 +10245,7 @@
         <v>3</v>
       </c>
       <c r="D13" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="E13" t="s">
         <v>311</v>
@@ -10259,7 +10259,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="B14">
         <v>166711</v>
@@ -10268,21 +10268,21 @@
         <v>4</v>
       </c>
       <c r="D14" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="E14" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="F14" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="G14" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="B15">
         <v>166755</v>
@@ -10291,13 +10291,13 @@
         <v>5</v>
       </c>
       <c r="D15" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="E15" t="s">
         <v>172</v>
       </c>
       <c r="F15" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="G15" t="s">
         <v>118</v>
@@ -10305,7 +10305,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="B16">
         <v>166757</v>
@@ -10314,21 +10314,21 @@
         <v>6</v>
       </c>
       <c r="D16" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="E16" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="F16" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="G16" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="B17">
         <v>167481</v>
@@ -10337,13 +10337,13 @@
         <v>7</v>
       </c>
       <c r="D17" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="E17" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="F17" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="G17" t="s">
         <v>114</v>
@@ -10351,7 +10351,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="B18">
         <v>167793</v>
@@ -10360,13 +10360,13 @@
         <v>8</v>
       </c>
       <c r="D18" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E18" t="s">
         <v>162</v>
       </c>
       <c r="F18" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="G18" t="s">
         <v>118</v>
@@ -10374,7 +10374,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="B19">
         <v>168287</v>
@@ -10383,21 +10383,21 @@
         <v>9</v>
       </c>
       <c r="D19" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="E19" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="F19" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="G19" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="B20">
         <v>166567</v>
@@ -10406,21 +10406,21 @@
         <v>1</v>
       </c>
       <c r="D20" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="E20" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="F20" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="G20" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="B21">
         <v>166538</v>
@@ -10429,21 +10429,21 @@
         <v>2</v>
       </c>
       <c r="D21" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="E21" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="F21" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="G21" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="B22">
         <v>166678</v>
@@ -10452,21 +10452,21 @@
         <v>3</v>
       </c>
       <c r="D22" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="E22" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="F22" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="G22" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="B23">
         <v>167682</v>
@@ -10475,21 +10475,21 @@
         <v>4</v>
       </c>
       <c r="D23" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="E23" t="s">
         <v>340</v>
       </c>
       <c r="F23" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="G23" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="B24">
         <v>166529</v>
@@ -10498,21 +10498,21 @@
         <v>5</v>
       </c>
       <c r="D24" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="E24" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="F24" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="G24" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="B25">
         <v>166472</v>
@@ -10521,21 +10521,21 @@
         <v>6</v>
       </c>
       <c r="D25" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="E25" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="F25" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="G25" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="B26">
         <v>166571</v>
@@ -10544,21 +10544,21 @@
         <v>7</v>
       </c>
       <c r="D26" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="E26" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="F26" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="G26" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="B27">
         <v>166575</v>
@@ -10567,13 +10567,13 @@
         <v>8</v>
       </c>
       <c r="D27" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="E27" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F27" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="G27" t="s">
         <v>118</v>
@@ -10581,7 +10581,7 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="B28">
         <v>166590</v>
@@ -10590,21 +10590,21 @@
         <v>9</v>
       </c>
       <c r="D28" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="E28" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="F28" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="G28" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="B29">
         <v>166598</v>
@@ -10613,21 +10613,21 @@
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="E29" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="F29" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="G29" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="B30">
         <v>166629</v>
@@ -10636,13 +10636,13 @@
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="E30" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="F30" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="G30" t="s">
         <v>118</v>
@@ -10650,7 +10650,7 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="B31">
         <v>166650</v>
@@ -10659,21 +10659,21 @@
         <v>3</v>
       </c>
       <c r="D31" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="E31" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="F31" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="G31" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="B32">
         <v>166657</v>
@@ -10682,13 +10682,13 @@
         <v>4</v>
       </c>
       <c r="D32" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="E32" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="F32" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="G32" t="s">
         <v>114</v>
@@ -10696,7 +10696,7 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="B33">
         <v>166687</v>
@@ -10705,21 +10705,21 @@
         <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="E33" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="F33" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="G33" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="B34">
         <v>166691</v>
@@ -10728,7 +10728,7 @@
         <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="E34" t="s">
         <v>336</v>
@@ -10742,7 +10742,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="B35">
         <v>166708</v>
@@ -10751,13 +10751,13 @@
         <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="E35" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="F35" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="G35" t="s">
         <v>118</v>
@@ -10765,7 +10765,7 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="B36">
         <v>166719</v>
@@ -10774,21 +10774,21 @@
         <v>8</v>
       </c>
       <c r="D36" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="E36" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="F36" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="G36" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B37">
         <v>166744</v>
@@ -10797,13 +10797,13 @@
         <v>9</v>
       </c>
       <c r="D37" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="E37" t="s">
         <v>322</v>
       </c>
       <c r="F37" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="G37" t="s">
         <v>118</v>
@@ -10811,7 +10811,7 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="B38">
         <v>166746</v>
@@ -10820,21 +10820,21 @@
         <v>1</v>
       </c>
       <c r="D38" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="E38" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="F38" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="G38" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="B39">
         <v>166753</v>
@@ -10843,21 +10843,21 @@
         <v>2</v>
       </c>
       <c r="D39" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="E39" t="s">
         <v>312</v>
       </c>
       <c r="F39" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="G39" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="B40">
         <v>166779</v>
@@ -10866,13 +10866,13 @@
         <v>3</v>
       </c>
       <c r="D40" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="E40" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="F40" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="G40" t="s">
         <v>118</v>
@@ -10880,7 +10880,7 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="B41">
         <v>166818</v>
@@ -10889,21 +10889,21 @@
         <v>4</v>
       </c>
       <c r="D41" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="E41" t="s">
         <v>84</v>
       </c>
       <c r="F41" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="G41" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="B42">
         <v>167482</v>
@@ -10912,13 +10912,13 @@
         <v>5</v>
       </c>
       <c r="D42" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="E42" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="F42" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="G42" t="s">
         <v>118</v>
@@ -10926,7 +10926,7 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="B43">
         <v>167812</v>
@@ -10935,13 +10935,13 @@
         <v>6</v>
       </c>
       <c r="D43" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="E43" t="s">
         <v>326</v>
       </c>
       <c r="F43" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="G43" t="s">
         <v>118</v>
@@ -10949,7 +10949,7 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="B44">
         <v>171332</v>
@@ -10958,16 +10958,16 @@
         <v>7</v>
       </c>
       <c r="D44" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="E44" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="F44" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="G44" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Program updated, author 363
</commit_message>
<xml_diff>
--- a/pm2022/pm2022.xlsx
+++ b/pm2022/pm2022.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/galli/Documents/OrgConferenze/21PisaMeeting/pisameet/pm2022/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06519633-1D65-684B-9144-B42DF361114C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7216461D-DE59-7B4C-B2FF-C1FF4EBEA6D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19360" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19360" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Program" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1505" uniqueCount="1190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1505" uniqueCount="1188">
   <si>
     <t>Session ID</t>
   </si>
@@ -3346,9 +3346,6 @@
     <t>Wu</t>
   </si>
   <si>
-    <t>Cammarata</t>
-  </si>
-  <si>
     <t>Gurgone</t>
   </si>
   <si>
@@ -3470,9 +3467,6 @@
   </si>
   <si>
     <t>Radboud University</t>
-  </si>
-  <si>
-    <t>Dipartimento di Ingegneria dell'Informazione - Università di Pisa</t>
   </si>
   <si>
     <t>Pavia U. &amp; INFN</t>
@@ -4037,10 +4031,10 @@
         <v>13</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>1164</v>
+        <v>1162</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>1169</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -4051,10 +4045,10 @@
         <v>14</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>1164</v>
+        <v>1162</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>1169</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -4065,10 +4059,10 @@
         <v>15</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1165</v>
+        <v>1163</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>1170</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -4079,10 +4073,10 @@
         <v>16</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>1165</v>
+        <v>1163</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>1170</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -4093,10 +4087,10 @@
         <v>17</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1166</v>
+        <v>1164</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>1171</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -4107,10 +4101,10 @@
         <v>18</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>1172</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -4121,10 +4115,10 @@
         <v>19</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>1172</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -4135,10 +4129,10 @@
         <v>20</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>1168</v>
+        <v>1166</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>1173</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -4149,10 +4143,10 @@
         <v>21</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>1168</v>
+        <v>1166</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>1173</v>
+        <v>1171</v>
       </c>
     </row>
   </sheetData>
@@ -4215,7 +4209,7 @@
         <v>1087</v>
       </c>
       <c r="G2" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -4238,7 +4232,7 @@
         <v>1088</v>
       </c>
       <c r="G3" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -4261,7 +4255,7 @@
         <v>1089</v>
       </c>
       <c r="G4" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -4284,7 +4278,7 @@
         <v>1090</v>
       </c>
       <c r="G5" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -4330,7 +4324,7 @@
         <v>1092</v>
       </c>
       <c r="G7" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -4376,7 +4370,7 @@
         <v>1094</v>
       </c>
       <c r="G9" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -4445,7 +4439,7 @@
         <v>1096</v>
       </c>
       <c r="G12" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -4468,7 +4462,7 @@
         <v>1097</v>
       </c>
       <c r="G13" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -4560,7 +4554,7 @@
         <v>1099</v>
       </c>
       <c r="G17" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
@@ -4583,7 +4577,7 @@
         <v>1100</v>
       </c>
       <c r="G18" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
@@ -4652,7 +4646,7 @@
         <v>1103</v>
       </c>
       <c r="G21" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -4675,7 +4669,7 @@
         <v>1104</v>
       </c>
       <c r="G22" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
@@ -4692,13 +4686,13 @@
         <v>1023</v>
       </c>
       <c r="E23" t="s">
-        <v>326</v>
+        <v>1078</v>
       </c>
       <c r="F23" t="s">
-        <v>1105</v>
+        <v>1119</v>
       </c>
       <c r="G23" t="s">
-        <v>1147</v>
+        <v>118</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
@@ -4718,10 +4712,10 @@
         <v>318</v>
       </c>
       <c r="F24" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
       <c r="G24" t="s">
-        <v>1148</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
@@ -4764,10 +4758,10 @@
         <v>1071</v>
       </c>
       <c r="F26" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="G26" t="s">
-        <v>1149</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
@@ -4810,10 +4804,10 @@
         <v>601</v>
       </c>
       <c r="F28" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="G28" t="s">
-        <v>1150</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
@@ -4833,10 +4827,10 @@
         <v>1072</v>
       </c>
       <c r="F29" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="G29" t="s">
-        <v>1151</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
@@ -4856,7 +4850,7 @@
         <v>326</v>
       </c>
       <c r="F30" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="G30" t="s">
         <v>118</v>
@@ -4879,7 +4873,7 @@
         <v>712</v>
       </c>
       <c r="F31" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="G31" t="s">
         <v>118</v>
@@ -4902,7 +4896,7 @@
         <v>1073</v>
       </c>
       <c r="F32" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="G32" t="s">
         <v>118</v>
@@ -4925,7 +4919,7 @@
         <v>1074</v>
       </c>
       <c r="F33" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="G33" t="s">
         <v>118</v>
@@ -4948,7 +4942,7 @@
         <v>719</v>
       </c>
       <c r="F34" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="G34" t="s">
         <v>118</v>
@@ -4968,13 +4962,13 @@
         <v>1035</v>
       </c>
       <c r="E35" t="s">
-        <v>1180</v>
+        <v>1178</v>
       </c>
       <c r="F35" t="s">
-        <v>1181</v>
+        <v>1179</v>
       </c>
       <c r="G35" t="s">
-        <v>1152</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
@@ -4994,7 +4988,7 @@
         <v>1073</v>
       </c>
       <c r="F36" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
       <c r="G36" t="s">
         <v>118</v>
@@ -5017,10 +5011,10 @@
         <v>172</v>
       </c>
       <c r="F37" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="G37" t="s">
-        <v>1153</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
@@ -5040,10 +5034,10 @@
         <v>1075</v>
       </c>
       <c r="F38" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
       <c r="G38" t="s">
-        <v>1154</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
@@ -5063,10 +5057,10 @@
         <v>1076</v>
       </c>
       <c r="F39" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="G39" t="s">
-        <v>1155</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
@@ -5086,7 +5080,7 @@
         <v>1077</v>
       </c>
       <c r="F40" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="G40" t="s">
         <v>118</v>
@@ -5109,7 +5103,7 @@
         <v>1078</v>
       </c>
       <c r="F41" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="G41" t="s">
         <v>118</v>
@@ -5132,10 +5126,10 @@
         <v>1079</v>
       </c>
       <c r="F42" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="G42" t="s">
-        <v>1156</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
@@ -5155,10 +5149,10 @@
         <v>712</v>
       </c>
       <c r="F43" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="G43" t="s">
-        <v>1157</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
@@ -5178,7 +5172,7 @@
         <v>1080</v>
       </c>
       <c r="F44" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="G44" t="s">
         <v>480</v>
@@ -5201,7 +5195,7 @@
         <v>1081</v>
       </c>
       <c r="F45" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="G45" t="s">
         <v>940</v>
@@ -5247,7 +5241,7 @@
         <v>708</v>
       </c>
       <c r="F47" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="G47" t="s">
         <v>118</v>
@@ -5270,7 +5264,7 @@
         <v>706</v>
       </c>
       <c r="F48" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="G48" t="s">
         <v>118</v>
@@ -5293,10 +5287,10 @@
         <v>1082</v>
       </c>
       <c r="F49" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="G49" t="s">
-        <v>1158</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
@@ -5316,10 +5310,10 @@
         <v>1083</v>
       </c>
       <c r="F50" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="G50" t="s">
-        <v>1159</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
@@ -5362,10 +5356,10 @@
         <v>306</v>
       </c>
       <c r="F52" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="G52" t="s">
-        <v>1160</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
@@ -5385,7 +5379,7 @@
         <v>1084</v>
       </c>
       <c r="F53" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="G53" t="s">
         <v>118</v>
@@ -5408,7 +5402,7 @@
         <v>881</v>
       </c>
       <c r="F54" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
       <c r="G54" t="s">
         <v>118</v>
@@ -5431,10 +5425,10 @@
         <v>1085</v>
       </c>
       <c r="F55" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
       <c r="G55" t="s">
-        <v>1161</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
@@ -5454,10 +5448,10 @@
         <v>1086</v>
       </c>
       <c r="F56" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="G56" t="s">
-        <v>1162</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
@@ -5477,7 +5471,7 @@
         <v>341</v>
       </c>
       <c r="F57" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="G57" t="s">
         <v>118</v>
@@ -5497,13 +5491,13 @@
         <v>1058</v>
       </c>
       <c r="E58" t="s">
-        <v>1186</v>
+        <v>1184</v>
       </c>
       <c r="F58" t="s">
-        <v>1185</v>
+        <v>1183</v>
       </c>
       <c r="G58" t="s">
-        <v>1163</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
@@ -5517,7 +5511,7 @@
         <v>12</v>
       </c>
       <c r="D59" t="s">
-        <v>1187</v>
+        <v>1185</v>
       </c>
       <c r="E59" t="s">
         <v>543</v>
@@ -7181,7 +7175,7 @@
         <v>877</v>
       </c>
       <c r="F30" t="s">
-        <v>1174</v>
+        <v>1172</v>
       </c>
       <c r="G30" t="s">
         <v>400</v>
@@ -7612,7 +7606,7 @@
         <v>6</v>
       </c>
       <c r="D49" t="s">
-        <v>1188</v>
+        <v>1186</v>
       </c>
       <c r="E49" t="s">
         <v>458</v>
@@ -8088,7 +8082,7 @@
         <v>15</v>
       </c>
       <c r="D20" t="s">
-        <v>1189</v>
+        <v>1187</v>
       </c>
       <c r="E20" t="s">
         <v>312</v>
@@ -8120,7 +8114,7 @@
         <v>478</v>
       </c>
       <c r="G21" t="s">
-        <v>1179</v>
+        <v>1177</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -8134,16 +8128,16 @@
         <v>17</v>
       </c>
       <c r="D22" t="s">
+        <v>1173</v>
+      </c>
+      <c r="E22" t="s">
+        <v>1174</v>
+      </c>
+      <c r="F22" t="s">
         <v>1175</v>
       </c>
-      <c r="E22" t="s">
+      <c r="G22" t="s">
         <v>1176</v>
-      </c>
-      <c r="F22" t="s">
-        <v>1177</v>
-      </c>
-      <c r="G22" t="s">
-        <v>1178</v>
       </c>
     </row>
   </sheetData>
@@ -8619,7 +8613,7 @@
         <v>564</v>
       </c>
       <c r="G20" t="s">
-        <v>1182</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -9266,10 +9260,10 @@
         <v>673</v>
       </c>
       <c r="E14" t="s">
-        <v>1183</v>
+        <v>1181</v>
       </c>
       <c r="F14" t="s">
-        <v>1184</v>
+        <v>1182</v>
       </c>
       <c r="G14" t="s">
         <v>118</v>

</xml_diff>

<commit_message>
Aggiunto 399 e 252
</commit_message>
<xml_diff>
--- a/pm2022/pm2022.xlsx
+++ b/pm2022/pm2022.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/galli/Documents/OrgConferenze/21PisaMeeting/pisameet/pm2022/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{755A24DD-3FDE-B842-BA11-0379498D879B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC768A8D-7575-F24D-A427-DDD3BBB4E33B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="220" yWindow="500" windowWidth="31720" windowHeight="18600" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="220" yWindow="500" windowWidth="31720" windowHeight="18600" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Program" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1446" uniqueCount="1162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1454" uniqueCount="1163">
   <si>
     <t>Session ID</t>
   </si>
@@ -3515,6 +3515,9 @@
   </si>
   <si>
     <t>University of Pisa and INFN - Pisa</t>
+  </si>
+  <si>
+    <t>Test beam results and future R&amp;D of the fibre-sampling Dual-Readout Calorimeter</t>
   </si>
 </sst>
 </file>
@@ -7425,7 +7428,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="3" width="12.6640625" customWidth="1"/>
@@ -7894,6 +7897,29 @@
         <v>476</v>
       </c>
     </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" s="2">
+        <v>252</v>
+      </c>
+      <c r="B21">
+        <v>172148</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21" t="s">
+        <v>420</v>
+      </c>
+      <c r="E21" t="s">
+        <v>439</v>
+      </c>
+      <c r="F21" t="s">
+        <v>452</v>
+      </c>
+      <c r="G21" t="s">
+        <v>468</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7901,7 +7927,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="3" width="12.6640625" customWidth="1"/>
@@ -8368,6 +8394,29 @@
       </c>
       <c r="G20" t="s">
         <v>1136</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" s="2">
+        <v>399</v>
+      </c>
+      <c r="B21">
+        <v>172147</v>
+      </c>
+      <c r="C21">
+        <v>20</v>
+      </c>
+      <c r="D21" t="s">
+        <v>1162</v>
+      </c>
+      <c r="E21" t="s">
+        <v>449</v>
+      </c>
+      <c r="F21" t="s">
+        <v>466</v>
+      </c>
+      <c r="G21" t="s">
+        <v>1156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>